<commit_message>
atualizando dados excel e carrossel
</commit_message>
<xml_diff>
--- a/LoteriasExcel/Lotofacil_edt2.xlsx
+++ b/LoteriasExcel/Lotofacil_edt2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Dropbox\! 000 ByPass\Pessoal\99_Loterias\0 - Loterias-Inteligentes\LoteriasExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EDCB27B-F5B4-4F66-B6A9-76A06A00045C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7464987B-B19E-4B52-8FFC-5A7A27FD9842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57585" yWindow="1395" windowWidth="18675" windowHeight="12840" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
+    <workbookView xWindow="66855" yWindow="810" windowWidth="18675" windowHeight="12840" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
   </bookViews>
   <sheets>
     <sheet name="LOTOFÁCIL" sheetId="3" r:id="rId1"/>
@@ -148,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -156,8 +156,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69BEFC42-DD13-4DE0-B2AD-D0F44AF8189C}">
-  <dimension ref="A1:P598"/>
+  <dimension ref="A1:P600"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="17" max="17" width="11.6640625" customWidth="1"/>
@@ -29638,752 +29636,852 @@
       </c>
     </row>
     <row r="584" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A584" s="5">
+      <c r="A584">
         <v>3654</v>
       </c>
-      <c r="B584" s="6">
-        <v>1</v>
-      </c>
-      <c r="C584" s="6">
-        <v>2</v>
-      </c>
-      <c r="D584" s="6">
-        <v>3</v>
-      </c>
-      <c r="E584" s="6">
-        <v>4</v>
-      </c>
-      <c r="F584" s="6">
-        <v>6</v>
-      </c>
-      <c r="G584" s="6">
-        <v>7</v>
-      </c>
-      <c r="H584" s="6">
-        <v>11</v>
-      </c>
-      <c r="I584" s="6">
-        <v>15</v>
-      </c>
-      <c r="J584" s="6">
-        <v>17</v>
-      </c>
-      <c r="K584" s="6">
-        <v>19</v>
-      </c>
-      <c r="L584" s="6">
-        <v>20</v>
-      </c>
-      <c r="M584" s="6">
-        <v>22</v>
-      </c>
-      <c r="N584" s="6">
-        <v>23</v>
-      </c>
-      <c r="O584" s="6">
-        <v>24</v>
-      </c>
-      <c r="P584" s="6">
+      <c r="B584">
+        <v>1</v>
+      </c>
+      <c r="C584">
+        <v>2</v>
+      </c>
+      <c r="D584">
+        <v>3</v>
+      </c>
+      <c r="E584">
+        <v>4</v>
+      </c>
+      <c r="F584">
+        <v>6</v>
+      </c>
+      <c r="G584">
+        <v>7</v>
+      </c>
+      <c r="H584">
+        <v>11</v>
+      </c>
+      <c r="I584">
+        <v>15</v>
+      </c>
+      <c r="J584">
+        <v>17</v>
+      </c>
+      <c r="K584">
+        <v>19</v>
+      </c>
+      <c r="L584">
+        <v>20</v>
+      </c>
+      <c r="M584">
+        <v>22</v>
+      </c>
+      <c r="N584">
+        <v>23</v>
+      </c>
+      <c r="O584">
+        <v>24</v>
+      </c>
+      <c r="P584">
         <v>25</v>
       </c>
     </row>
     <row r="585" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A585" s="5">
+      <c r="A585">
         <v>3655</v>
       </c>
-      <c r="B585" s="6">
-        <v>1</v>
-      </c>
-      <c r="C585" s="6">
-        <v>2</v>
-      </c>
-      <c r="D585" s="6">
-        <v>4</v>
-      </c>
-      <c r="E585" s="6">
-        <v>5</v>
-      </c>
-      <c r="F585" s="6">
-        <v>6</v>
-      </c>
-      <c r="G585" s="6">
-        <v>10</v>
-      </c>
-      <c r="H585" s="6">
-        <v>11</v>
-      </c>
-      <c r="I585" s="6">
-        <v>12</v>
-      </c>
-      <c r="J585" s="6">
-        <v>17</v>
-      </c>
-      <c r="K585" s="6">
-        <v>18</v>
-      </c>
-      <c r="L585" s="6">
-        <v>19</v>
-      </c>
-      <c r="M585" s="6">
-        <v>21</v>
-      </c>
-      <c r="N585" s="6">
-        <v>22</v>
-      </c>
-      <c r="O585" s="6">
-        <v>23</v>
-      </c>
-      <c r="P585" s="6">
+      <c r="B585">
+        <v>1</v>
+      </c>
+      <c r="C585">
+        <v>2</v>
+      </c>
+      <c r="D585">
+        <v>4</v>
+      </c>
+      <c r="E585">
+        <v>5</v>
+      </c>
+      <c r="F585">
+        <v>6</v>
+      </c>
+      <c r="G585">
+        <v>10</v>
+      </c>
+      <c r="H585">
+        <v>11</v>
+      </c>
+      <c r="I585">
+        <v>12</v>
+      </c>
+      <c r="J585">
+        <v>17</v>
+      </c>
+      <c r="K585">
+        <v>18</v>
+      </c>
+      <c r="L585">
+        <v>19</v>
+      </c>
+      <c r="M585">
+        <v>21</v>
+      </c>
+      <c r="N585">
+        <v>22</v>
+      </c>
+      <c r="O585">
+        <v>23</v>
+      </c>
+      <c r="P585">
         <v>24</v>
       </c>
     </row>
     <row r="586" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A586" s="5">
+      <c r="A586">
         <v>3656</v>
       </c>
-      <c r="B586" s="6">
-        <v>3</v>
-      </c>
-      <c r="C586" s="6">
-        <v>4</v>
-      </c>
-      <c r="D586" s="6">
-        <v>6</v>
-      </c>
-      <c r="E586" s="6">
-        <v>7</v>
-      </c>
-      <c r="F586" s="6">
-        <v>8</v>
-      </c>
-      <c r="G586" s="6">
-        <v>11</v>
-      </c>
-      <c r="H586" s="6">
-        <v>12</v>
-      </c>
-      <c r="I586" s="6">
-        <v>14</v>
-      </c>
-      <c r="J586" s="6">
-        <v>15</v>
-      </c>
-      <c r="K586" s="6">
-        <v>18</v>
-      </c>
-      <c r="L586" s="6">
-        <v>19</v>
-      </c>
-      <c r="M586" s="6">
-        <v>20</v>
-      </c>
-      <c r="N586" s="6">
-        <v>21</v>
-      </c>
-      <c r="O586" s="6">
-        <v>24</v>
-      </c>
-      <c r="P586" s="6">
+      <c r="B586">
+        <v>3</v>
+      </c>
+      <c r="C586">
+        <v>4</v>
+      </c>
+      <c r="D586">
+        <v>6</v>
+      </c>
+      <c r="E586">
+        <v>7</v>
+      </c>
+      <c r="F586">
+        <v>8</v>
+      </c>
+      <c r="G586">
+        <v>11</v>
+      </c>
+      <c r="H586">
+        <v>12</v>
+      </c>
+      <c r="I586">
+        <v>14</v>
+      </c>
+      <c r="J586">
+        <v>15</v>
+      </c>
+      <c r="K586">
+        <v>18</v>
+      </c>
+      <c r="L586">
+        <v>19</v>
+      </c>
+      <c r="M586">
+        <v>20</v>
+      </c>
+      <c r="N586">
+        <v>21</v>
+      </c>
+      <c r="O586">
+        <v>24</v>
+      </c>
+      <c r="P586">
         <v>25</v>
       </c>
     </row>
     <row r="587" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A587" s="5">
+      <c r="A587">
         <v>3657</v>
       </c>
-      <c r="B587" s="6">
-        <v>1</v>
-      </c>
-      <c r="C587" s="6">
-        <v>2</v>
-      </c>
-      <c r="D587" s="6">
-        <v>4</v>
-      </c>
-      <c r="E587" s="6">
-        <v>7</v>
-      </c>
-      <c r="F587" s="6">
-        <v>8</v>
-      </c>
-      <c r="G587" s="6">
-        <v>10</v>
-      </c>
-      <c r="H587" s="6">
-        <v>12</v>
-      </c>
-      <c r="I587" s="6">
-        <v>13</v>
-      </c>
-      <c r="J587" s="6">
-        <v>17</v>
-      </c>
-      <c r="K587" s="6">
-        <v>18</v>
-      </c>
-      <c r="L587" s="6">
-        <v>19</v>
-      </c>
-      <c r="M587" s="6">
-        <v>20</v>
-      </c>
-      <c r="N587" s="6">
-        <v>22</v>
-      </c>
-      <c r="O587" s="6">
-        <v>23</v>
-      </c>
-      <c r="P587" s="6">
+      <c r="B587">
+        <v>1</v>
+      </c>
+      <c r="C587">
+        <v>2</v>
+      </c>
+      <c r="D587">
+        <v>4</v>
+      </c>
+      <c r="E587">
+        <v>7</v>
+      </c>
+      <c r="F587">
+        <v>8</v>
+      </c>
+      <c r="G587">
+        <v>10</v>
+      </c>
+      <c r="H587">
+        <v>12</v>
+      </c>
+      <c r="I587">
+        <v>13</v>
+      </c>
+      <c r="J587">
+        <v>17</v>
+      </c>
+      <c r="K587">
+        <v>18</v>
+      </c>
+      <c r="L587">
+        <v>19</v>
+      </c>
+      <c r="M587">
+        <v>20</v>
+      </c>
+      <c r="N587">
+        <v>22</v>
+      </c>
+      <c r="O587">
+        <v>23</v>
+      </c>
+      <c r="P587">
         <v>24</v>
       </c>
     </row>
     <row r="588" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A588" s="5">
+      <c r="A588">
         <v>3658</v>
       </c>
-      <c r="B588" s="6">
-        <v>2</v>
-      </c>
-      <c r="C588" s="6">
-        <v>3</v>
-      </c>
-      <c r="D588" s="6">
-        <v>4</v>
-      </c>
-      <c r="E588" s="6">
-        <v>5</v>
-      </c>
-      <c r="F588" s="6">
-        <v>9</v>
-      </c>
-      <c r="G588" s="6">
-        <v>10</v>
-      </c>
-      <c r="H588" s="6">
-        <v>11</v>
-      </c>
-      <c r="I588" s="6">
-        <v>12</v>
-      </c>
-      <c r="J588" s="6">
-        <v>13</v>
-      </c>
-      <c r="K588" s="6">
-        <v>16</v>
-      </c>
-      <c r="L588" s="6">
-        <v>18</v>
-      </c>
-      <c r="M588" s="6">
-        <v>20</v>
-      </c>
-      <c r="N588" s="6">
-        <v>22</v>
-      </c>
-      <c r="O588" s="6">
-        <v>23</v>
-      </c>
-      <c r="P588" s="6">
+      <c r="B588">
+        <v>2</v>
+      </c>
+      <c r="C588">
+        <v>3</v>
+      </c>
+      <c r="D588">
+        <v>4</v>
+      </c>
+      <c r="E588">
+        <v>5</v>
+      </c>
+      <c r="F588">
+        <v>9</v>
+      </c>
+      <c r="G588">
+        <v>10</v>
+      </c>
+      <c r="H588">
+        <v>11</v>
+      </c>
+      <c r="I588">
+        <v>12</v>
+      </c>
+      <c r="J588">
+        <v>13</v>
+      </c>
+      <c r="K588">
+        <v>16</v>
+      </c>
+      <c r="L588">
+        <v>18</v>
+      </c>
+      <c r="M588">
+        <v>20</v>
+      </c>
+      <c r="N588">
+        <v>22</v>
+      </c>
+      <c r="O588">
+        <v>23</v>
+      </c>
+      <c r="P588">
         <v>24</v>
       </c>
     </row>
     <row r="589" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A589" s="5">
+      <c r="A589">
         <v>3659</v>
       </c>
-      <c r="B589" s="6">
-        <v>3</v>
-      </c>
-      <c r="C589" s="6">
-        <v>5</v>
-      </c>
-      <c r="D589" s="6">
-        <v>6</v>
-      </c>
-      <c r="E589" s="6">
-        <v>7</v>
-      </c>
-      <c r="F589" s="6">
-        <v>8</v>
-      </c>
-      <c r="G589" s="6">
-        <v>9</v>
-      </c>
-      <c r="H589" s="6">
-        <v>10</v>
-      </c>
-      <c r="I589" s="6">
-        <v>11</v>
-      </c>
-      <c r="J589" s="6">
-        <v>13</v>
-      </c>
-      <c r="K589" s="6">
-        <v>14</v>
-      </c>
-      <c r="L589" s="6">
-        <v>15</v>
-      </c>
-      <c r="M589" s="6">
-        <v>16</v>
-      </c>
-      <c r="N589" s="6">
-        <v>17</v>
-      </c>
-      <c r="O589" s="6">
-        <v>23</v>
-      </c>
-      <c r="P589" s="6">
+      <c r="B589">
+        <v>3</v>
+      </c>
+      <c r="C589">
+        <v>5</v>
+      </c>
+      <c r="D589">
+        <v>6</v>
+      </c>
+      <c r="E589">
+        <v>7</v>
+      </c>
+      <c r="F589">
+        <v>8</v>
+      </c>
+      <c r="G589">
+        <v>9</v>
+      </c>
+      <c r="H589">
+        <v>10</v>
+      </c>
+      <c r="I589">
+        <v>11</v>
+      </c>
+      <c r="J589">
+        <v>13</v>
+      </c>
+      <c r="K589">
+        <v>14</v>
+      </c>
+      <c r="L589">
+        <v>15</v>
+      </c>
+      <c r="M589">
+        <v>16</v>
+      </c>
+      <c r="N589">
+        <v>17</v>
+      </c>
+      <c r="O589">
+        <v>23</v>
+      </c>
+      <c r="P589">
         <v>25</v>
       </c>
     </row>
     <row r="590" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A590" s="5">
+      <c r="A590">
         <v>3660</v>
       </c>
-      <c r="B590" s="6">
-        <v>1</v>
-      </c>
-      <c r="C590" s="6">
-        <v>2</v>
-      </c>
-      <c r="D590" s="6">
-        <v>5</v>
-      </c>
-      <c r="E590" s="6">
-        <v>6</v>
-      </c>
-      <c r="F590" s="6">
-        <v>7</v>
-      </c>
-      <c r="G590" s="6">
-        <v>8</v>
-      </c>
-      <c r="H590" s="6">
-        <v>10</v>
-      </c>
-      <c r="I590" s="6">
-        <v>11</v>
-      </c>
-      <c r="J590" s="6">
-        <v>12</v>
-      </c>
-      <c r="K590" s="6">
-        <v>14</v>
-      </c>
-      <c r="L590" s="6">
-        <v>17</v>
-      </c>
-      <c r="M590" s="6">
-        <v>18</v>
-      </c>
-      <c r="N590" s="6">
-        <v>22</v>
-      </c>
-      <c r="O590" s="6">
-        <v>23</v>
-      </c>
-      <c r="P590" s="6">
+      <c r="B590">
+        <v>1</v>
+      </c>
+      <c r="C590">
+        <v>2</v>
+      </c>
+      <c r="D590">
+        <v>5</v>
+      </c>
+      <c r="E590">
+        <v>6</v>
+      </c>
+      <c r="F590">
+        <v>7</v>
+      </c>
+      <c r="G590">
+        <v>8</v>
+      </c>
+      <c r="H590">
+        <v>10</v>
+      </c>
+      <c r="I590">
+        <v>11</v>
+      </c>
+      <c r="J590">
+        <v>12</v>
+      </c>
+      <c r="K590">
+        <v>14</v>
+      </c>
+      <c r="L590">
+        <v>17</v>
+      </c>
+      <c r="M590">
+        <v>18</v>
+      </c>
+      <c r="N590">
+        <v>22</v>
+      </c>
+      <c r="O590">
+        <v>23</v>
+      </c>
+      <c r="P590">
         <v>24</v>
       </c>
     </row>
     <row r="591" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A591" s="5">
+      <c r="A591">
         <v>3661</v>
       </c>
-      <c r="B591" s="6">
-        <v>2</v>
-      </c>
-      <c r="C591" s="6">
-        <v>3</v>
-      </c>
-      <c r="D591" s="6">
-        <v>4</v>
-      </c>
-      <c r="E591" s="6">
-        <v>5</v>
-      </c>
-      <c r="F591" s="6">
-        <v>6</v>
-      </c>
-      <c r="G591" s="6">
-        <v>7</v>
-      </c>
-      <c r="H591" s="6">
-        <v>8</v>
-      </c>
-      <c r="I591" s="6">
-        <v>10</v>
-      </c>
-      <c r="J591" s="6">
-        <v>12</v>
-      </c>
-      <c r="K591" s="6">
-        <v>14</v>
-      </c>
-      <c r="L591" s="6">
-        <v>15</v>
-      </c>
-      <c r="M591" s="6">
-        <v>19</v>
-      </c>
-      <c r="N591" s="6">
-        <v>21</v>
-      </c>
-      <c r="O591" s="6">
-        <v>23</v>
-      </c>
-      <c r="P591" s="6">
+      <c r="B591">
+        <v>2</v>
+      </c>
+      <c r="C591">
+        <v>3</v>
+      </c>
+      <c r="D591">
+        <v>4</v>
+      </c>
+      <c r="E591">
+        <v>5</v>
+      </c>
+      <c r="F591">
+        <v>6</v>
+      </c>
+      <c r="G591">
+        <v>7</v>
+      </c>
+      <c r="H591">
+        <v>8</v>
+      </c>
+      <c r="I591">
+        <v>10</v>
+      </c>
+      <c r="J591">
+        <v>12</v>
+      </c>
+      <c r="K591">
+        <v>14</v>
+      </c>
+      <c r="L591">
+        <v>15</v>
+      </c>
+      <c r="M591">
+        <v>19</v>
+      </c>
+      <c r="N591">
+        <v>21</v>
+      </c>
+      <c r="O591">
+        <v>23</v>
+      </c>
+      <c r="P591">
         <v>24</v>
       </c>
     </row>
     <row r="592" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A592" s="5">
+      <c r="A592">
         <v>3662</v>
       </c>
-      <c r="B592" s="6">
-        <v>4</v>
-      </c>
-      <c r="C592" s="6">
-        <v>5</v>
-      </c>
-      <c r="D592" s="6">
-        <v>6</v>
-      </c>
-      <c r="E592" s="6">
-        <v>7</v>
-      </c>
-      <c r="F592" s="6">
-        <v>8</v>
-      </c>
-      <c r="G592" s="6">
-        <v>9</v>
-      </c>
-      <c r="H592" s="6">
-        <v>10</v>
-      </c>
-      <c r="I592" s="6">
-        <v>11</v>
-      </c>
-      <c r="J592" s="6">
-        <v>12</v>
-      </c>
-      <c r="K592" s="6">
-        <v>13</v>
-      </c>
-      <c r="L592" s="6">
-        <v>15</v>
-      </c>
-      <c r="M592" s="6">
-        <v>18</v>
-      </c>
-      <c r="N592" s="6">
-        <v>20</v>
-      </c>
-      <c r="O592" s="6">
-        <v>23</v>
-      </c>
-      <c r="P592" s="6">
+      <c r="B592">
+        <v>4</v>
+      </c>
+      <c r="C592">
+        <v>5</v>
+      </c>
+      <c r="D592">
+        <v>6</v>
+      </c>
+      <c r="E592">
+        <v>7</v>
+      </c>
+      <c r="F592">
+        <v>8</v>
+      </c>
+      <c r="G592">
+        <v>9</v>
+      </c>
+      <c r="H592">
+        <v>10</v>
+      </c>
+      <c r="I592">
+        <v>11</v>
+      </c>
+      <c r="J592">
+        <v>12</v>
+      </c>
+      <c r="K592">
+        <v>13</v>
+      </c>
+      <c r="L592">
+        <v>15</v>
+      </c>
+      <c r="M592">
+        <v>18</v>
+      </c>
+      <c r="N592">
+        <v>20</v>
+      </c>
+      <c r="O592">
+        <v>23</v>
+      </c>
+      <c r="P592">
         <v>25</v>
       </c>
     </row>
     <row r="593" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A593" s="5">
+      <c r="A593">
         <v>3663</v>
       </c>
-      <c r="B593" s="6">
-        <v>1</v>
-      </c>
-      <c r="C593" s="6">
-        <v>3</v>
-      </c>
-      <c r="D593" s="6">
-        <v>4</v>
-      </c>
-      <c r="E593" s="6">
-        <v>5</v>
-      </c>
-      <c r="F593" s="6">
-        <v>6</v>
-      </c>
-      <c r="G593" s="6">
-        <v>10</v>
-      </c>
-      <c r="H593" s="6">
-        <v>12</v>
-      </c>
-      <c r="I593" s="6">
-        <v>14</v>
-      </c>
-      <c r="J593" s="6">
-        <v>17</v>
-      </c>
-      <c r="K593" s="6">
-        <v>19</v>
-      </c>
-      <c r="L593" s="6">
-        <v>20</v>
-      </c>
-      <c r="M593" s="6">
-        <v>22</v>
-      </c>
-      <c r="N593" s="6">
-        <v>23</v>
-      </c>
-      <c r="O593" s="6">
-        <v>24</v>
-      </c>
-      <c r="P593" s="6">
+      <c r="B593">
+        <v>1</v>
+      </c>
+      <c r="C593">
+        <v>3</v>
+      </c>
+      <c r="D593">
+        <v>4</v>
+      </c>
+      <c r="E593">
+        <v>5</v>
+      </c>
+      <c r="F593">
+        <v>6</v>
+      </c>
+      <c r="G593">
+        <v>10</v>
+      </c>
+      <c r="H593">
+        <v>12</v>
+      </c>
+      <c r="I593">
+        <v>14</v>
+      </c>
+      <c r="J593">
+        <v>17</v>
+      </c>
+      <c r="K593">
+        <v>19</v>
+      </c>
+      <c r="L593">
+        <v>20</v>
+      </c>
+      <c r="M593">
+        <v>22</v>
+      </c>
+      <c r="N593">
+        <v>23</v>
+      </c>
+      <c r="O593">
+        <v>24</v>
+      </c>
+      <c r="P593">
         <v>25</v>
       </c>
     </row>
     <row r="594" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A594" s="5">
+      <c r="A594">
         <v>3664</v>
       </c>
-      <c r="B594" s="6">
-        <v>1</v>
-      </c>
-      <c r="C594" s="6">
-        <v>2</v>
-      </c>
-      <c r="D594" s="6">
-        <v>4</v>
-      </c>
-      <c r="E594" s="6">
-        <v>5</v>
-      </c>
-      <c r="F594" s="6">
-        <v>6</v>
-      </c>
-      <c r="G594" s="6">
-        <v>7</v>
-      </c>
-      <c r="H594" s="6">
-        <v>10</v>
-      </c>
-      <c r="I594" s="6">
-        <v>11</v>
-      </c>
-      <c r="J594" s="6">
-        <v>12</v>
-      </c>
-      <c r="K594" s="6">
-        <v>16</v>
-      </c>
-      <c r="L594" s="6">
-        <v>18</v>
-      </c>
-      <c r="M594" s="6">
-        <v>19</v>
-      </c>
-      <c r="N594" s="6">
-        <v>20</v>
-      </c>
-      <c r="O594" s="6">
-        <v>22</v>
-      </c>
-      <c r="P594" s="6">
+      <c r="B594">
+        <v>1</v>
+      </c>
+      <c r="C594">
+        <v>2</v>
+      </c>
+      <c r="D594">
+        <v>4</v>
+      </c>
+      <c r="E594">
+        <v>5</v>
+      </c>
+      <c r="F594">
+        <v>6</v>
+      </c>
+      <c r="G594">
+        <v>7</v>
+      </c>
+      <c r="H594">
+        <v>10</v>
+      </c>
+      <c r="I594">
+        <v>11</v>
+      </c>
+      <c r="J594">
+        <v>12</v>
+      </c>
+      <c r="K594">
+        <v>16</v>
+      </c>
+      <c r="L594">
+        <v>18</v>
+      </c>
+      <c r="M594">
+        <v>19</v>
+      </c>
+      <c r="N594">
+        <v>20</v>
+      </c>
+      <c r="O594">
+        <v>22</v>
+      </c>
+      <c r="P594">
         <v>23</v>
       </c>
     </row>
     <row r="595" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A595" s="5">
+      <c r="A595">
         <v>3665</v>
       </c>
-      <c r="B595" s="6">
-        <v>1</v>
-      </c>
-      <c r="C595" s="6">
-        <v>2</v>
-      </c>
-      <c r="D595" s="6">
-        <v>3</v>
-      </c>
-      <c r="E595" s="6">
-        <v>5</v>
-      </c>
-      <c r="F595" s="6">
-        <v>6</v>
-      </c>
-      <c r="G595" s="6">
-        <v>7</v>
-      </c>
-      <c r="H595" s="6">
-        <v>9</v>
-      </c>
-      <c r="I595" s="6">
-        <v>10</v>
-      </c>
-      <c r="J595" s="6">
-        <v>11</v>
-      </c>
-      <c r="K595" s="6">
-        <v>13</v>
-      </c>
-      <c r="L595" s="6">
-        <v>16</v>
-      </c>
-      <c r="M595" s="6">
-        <v>18</v>
-      </c>
-      <c r="N595" s="6">
-        <v>22</v>
-      </c>
-      <c r="O595" s="6">
-        <v>23</v>
-      </c>
-      <c r="P595" s="6">
+      <c r="B595">
+        <v>1</v>
+      </c>
+      <c r="C595">
+        <v>2</v>
+      </c>
+      <c r="D595">
+        <v>3</v>
+      </c>
+      <c r="E595">
+        <v>5</v>
+      </c>
+      <c r="F595">
+        <v>6</v>
+      </c>
+      <c r="G595">
+        <v>7</v>
+      </c>
+      <c r="H595">
+        <v>9</v>
+      </c>
+      <c r="I595">
+        <v>10</v>
+      </c>
+      <c r="J595">
+        <v>11</v>
+      </c>
+      <c r="K595">
+        <v>13</v>
+      </c>
+      <c r="L595">
+        <v>16</v>
+      </c>
+      <c r="M595">
+        <v>18</v>
+      </c>
+      <c r="N595">
+        <v>22</v>
+      </c>
+      <c r="O595">
+        <v>23</v>
+      </c>
+      <c r="P595">
         <v>25</v>
       </c>
     </row>
     <row r="596" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A596" s="5">
+      <c r="A596">
         <v>3666</v>
       </c>
-      <c r="B596" s="6">
-        <v>1</v>
-      </c>
-      <c r="C596" s="6">
-        <v>4</v>
-      </c>
-      <c r="D596" s="6">
-        <v>6</v>
-      </c>
-      <c r="E596" s="6">
-        <v>7</v>
-      </c>
-      <c r="F596" s="6">
-        <v>9</v>
-      </c>
-      <c r="G596" s="6">
-        <v>12</v>
-      </c>
-      <c r="H596" s="6">
-        <v>14</v>
-      </c>
-      <c r="I596" s="6">
-        <v>15</v>
-      </c>
-      <c r="J596" s="6">
-        <v>16</v>
-      </c>
-      <c r="K596" s="6">
-        <v>17</v>
-      </c>
-      <c r="L596" s="6">
-        <v>19</v>
-      </c>
-      <c r="M596" s="6">
-        <v>20</v>
-      </c>
-      <c r="N596" s="6">
-        <v>21</v>
-      </c>
-      <c r="O596" s="6">
-        <v>22</v>
-      </c>
-      <c r="P596" s="6">
+      <c r="B596">
+        <v>1</v>
+      </c>
+      <c r="C596">
+        <v>4</v>
+      </c>
+      <c r="D596">
+        <v>6</v>
+      </c>
+      <c r="E596">
+        <v>7</v>
+      </c>
+      <c r="F596">
+        <v>9</v>
+      </c>
+      <c r="G596">
+        <v>12</v>
+      </c>
+      <c r="H596">
+        <v>14</v>
+      </c>
+      <c r="I596">
+        <v>15</v>
+      </c>
+      <c r="J596">
+        <v>16</v>
+      </c>
+      <c r="K596">
+        <v>17</v>
+      </c>
+      <c r="L596">
+        <v>19</v>
+      </c>
+      <c r="M596">
+        <v>20</v>
+      </c>
+      <c r="N596">
+        <v>21</v>
+      </c>
+      <c r="O596">
+        <v>22</v>
+      </c>
+      <c r="P596">
         <v>23</v>
       </c>
     </row>
     <row r="597" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A597" s="5">
+      <c r="A597">
         <v>3667</v>
       </c>
-      <c r="B597" s="6">
-        <v>1</v>
-      </c>
-      <c r="C597" s="6">
-        <v>3</v>
-      </c>
-      <c r="D597" s="6">
-        <v>4</v>
-      </c>
-      <c r="E597" s="6">
-        <v>5</v>
-      </c>
-      <c r="F597" s="6">
-        <v>6</v>
-      </c>
-      <c r="G597" s="6">
-        <v>7</v>
-      </c>
-      <c r="H597" s="6">
-        <v>9</v>
-      </c>
-      <c r="I597" s="6">
-        <v>11</v>
-      </c>
-      <c r="J597" s="6">
-        <v>14</v>
-      </c>
-      <c r="K597" s="6">
-        <v>15</v>
-      </c>
-      <c r="L597" s="6">
-        <v>19</v>
-      </c>
-      <c r="M597" s="6">
-        <v>21</v>
-      </c>
-      <c r="N597" s="6">
-        <v>22</v>
-      </c>
-      <c r="O597" s="6">
-        <v>23</v>
-      </c>
-      <c r="P597" s="6">
+      <c r="B597">
+        <v>1</v>
+      </c>
+      <c r="C597">
+        <v>3</v>
+      </c>
+      <c r="D597">
+        <v>4</v>
+      </c>
+      <c r="E597">
+        <v>5</v>
+      </c>
+      <c r="F597">
+        <v>6</v>
+      </c>
+      <c r="G597">
+        <v>7</v>
+      </c>
+      <c r="H597">
+        <v>9</v>
+      </c>
+      <c r="I597">
+        <v>11</v>
+      </c>
+      <c r="J597">
+        <v>14</v>
+      </c>
+      <c r="K597">
+        <v>15</v>
+      </c>
+      <c r="L597">
+        <v>19</v>
+      </c>
+      <c r="M597">
+        <v>21</v>
+      </c>
+      <c r="N597">
+        <v>22</v>
+      </c>
+      <c r="O597">
+        <v>23</v>
+      </c>
+      <c r="P597">
         <v>25</v>
       </c>
     </row>
     <row r="598" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A598" s="5">
+      <c r="A598">
         <v>3668</v>
       </c>
-      <c r="B598" s="6">
-        <v>1</v>
-      </c>
-      <c r="C598" s="6">
-        <v>2</v>
-      </c>
-      <c r="D598" s="6">
-        <v>3</v>
-      </c>
-      <c r="E598" s="6">
-        <v>5</v>
-      </c>
-      <c r="F598" s="6">
-        <v>7</v>
-      </c>
-      <c r="G598" s="6">
-        <v>8</v>
-      </c>
-      <c r="H598" s="6">
-        <v>9</v>
-      </c>
-      <c r="I598" s="6">
-        <v>10</v>
-      </c>
-      <c r="J598" s="6">
-        <v>11</v>
-      </c>
-      <c r="K598" s="6">
-        <v>13</v>
-      </c>
-      <c r="L598" s="6">
-        <v>15</v>
-      </c>
-      <c r="M598" s="6">
-        <v>17</v>
-      </c>
-      <c r="N598" s="6">
-        <v>18</v>
-      </c>
-      <c r="O598" s="6">
-        <v>21</v>
-      </c>
-      <c r="P598" s="6">
+      <c r="B598">
+        <v>1</v>
+      </c>
+      <c r="C598">
+        <v>2</v>
+      </c>
+      <c r="D598">
+        <v>3</v>
+      </c>
+      <c r="E598">
+        <v>5</v>
+      </c>
+      <c r="F598">
+        <v>7</v>
+      </c>
+      <c r="G598">
+        <v>8</v>
+      </c>
+      <c r="H598">
+        <v>9</v>
+      </c>
+      <c r="I598">
+        <v>10</v>
+      </c>
+      <c r="J598">
+        <v>11</v>
+      </c>
+      <c r="K598">
+        <v>13</v>
+      </c>
+      <c r="L598">
+        <v>15</v>
+      </c>
+      <c r="M598">
+        <v>17</v>
+      </c>
+      <c r="N598">
+        <v>18</v>
+      </c>
+      <c r="O598">
+        <v>21</v>
+      </c>
+      <c r="P598">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="599" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A599">
+        <v>3669</v>
+      </c>
+      <c r="B599">
+        <v>2</v>
+      </c>
+      <c r="C599">
+        <v>3</v>
+      </c>
+      <c r="D599">
+        <v>4</v>
+      </c>
+      <c r="E599">
+        <v>5</v>
+      </c>
+      <c r="F599">
+        <v>8</v>
+      </c>
+      <c r="G599">
+        <v>9</v>
+      </c>
+      <c r="H599">
+        <v>10</v>
+      </c>
+      <c r="I599">
+        <v>11</v>
+      </c>
+      <c r="J599">
+        <v>12</v>
+      </c>
+      <c r="K599">
+        <v>15</v>
+      </c>
+      <c r="L599">
+        <v>16</v>
+      </c>
+      <c r="M599">
+        <v>17</v>
+      </c>
+      <c r="N599">
+        <v>22</v>
+      </c>
+      <c r="O599">
+        <v>23</v>
+      </c>
+      <c r="P599">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="600" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A600">
+        <v>3670</v>
+      </c>
+      <c r="B600">
+        <v>1</v>
+      </c>
+      <c r="C600">
+        <v>2</v>
+      </c>
+      <c r="D600">
+        <v>3</v>
+      </c>
+      <c r="E600">
+        <v>5</v>
+      </c>
+      <c r="F600">
+        <v>6</v>
+      </c>
+      <c r="G600">
+        <v>10</v>
+      </c>
+      <c r="H600">
+        <v>11</v>
+      </c>
+      <c r="I600">
+        <v>14</v>
+      </c>
+      <c r="J600">
+        <v>15</v>
+      </c>
+      <c r="K600">
+        <v>17</v>
+      </c>
+      <c r="L600">
+        <v>18</v>
+      </c>
+      <c r="M600">
+        <v>19</v>
+      </c>
+      <c r="N600">
+        <v>21</v>
+      </c>
+      <c r="O600">
+        <v>23</v>
+      </c>
+      <c r="P600">
         <v>24</v>
       </c>
     </row>
@@ -30393,15 +30491,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C92CDE8829F3C7438DCCB0991C30EAAE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36cf41eecaf38ba1d849a0c8dd067090">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="3e38fcf2-aa96-4a2c-865b-c3abba01ba51" xmlns:ns3="4455b8ba-124f-46d5-aaaa-9813efd83d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="023f68b2d27389a617bf935a3f0e17ad" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -30569,6 +30658,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -30580,14 +30678,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B637BD-743B-452C-A85E-33AF8B93F052}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C5B8C5-4575-4105-836C-9C4A6674A14B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -30607,6 +30697,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B637BD-743B-452C-A85E-33AF8B93F052}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0328C38C-FE97-4791-8469-4B5D9CCC5D08}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
atualizando excels e carrossel
</commit_message>
<xml_diff>
--- a/LoteriasExcel/Lotofacil_edt2.xlsx
+++ b/LoteriasExcel/Lotofacil_edt2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Dropbox\! 000 ByPass\Pessoal\99_Loterias\0 - Loterias-Inteligentes\LoteriasExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8086D3D-92C3-4C3A-A6FD-921F5490B713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C5D69A-20AE-437B-87DF-72A535F80DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8190" yWindow="1493" windowWidth="19590" windowHeight="12509" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
+    <workbookView xWindow="59010" yWindow="120" windowWidth="15285" windowHeight="13365" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
   </bookViews>
   <sheets>
     <sheet name="LOTOFÁCIL" sheetId="3" r:id="rId1"/>
@@ -476,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69BEFC42-DD13-4DE0-B2AD-D0F44AF8189C}">
-  <dimension ref="A1:P609"/>
+  <dimension ref="A1:P646"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="17" max="17" width="11.6640625" customWidth="1"/>
@@ -30935,12 +30935,1871 @@
         <v>24</v>
       </c>
     </row>
+    <row r="610" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A610">
+        <v>3680</v>
+      </c>
+      <c r="B610">
+        <v>1</v>
+      </c>
+      <c r="C610">
+        <v>2</v>
+      </c>
+      <c r="D610">
+        <v>3</v>
+      </c>
+      <c r="E610">
+        <v>4</v>
+      </c>
+      <c r="F610">
+        <v>5</v>
+      </c>
+      <c r="G610">
+        <v>7</v>
+      </c>
+      <c r="H610">
+        <v>8</v>
+      </c>
+      <c r="I610">
+        <v>9</v>
+      </c>
+      <c r="J610">
+        <v>11</v>
+      </c>
+      <c r="K610">
+        <v>15</v>
+      </c>
+      <c r="L610">
+        <v>16</v>
+      </c>
+      <c r="M610">
+        <v>19</v>
+      </c>
+      <c r="N610">
+        <v>22</v>
+      </c>
+      <c r="O610">
+        <v>24</v>
+      </c>
+      <c r="P610">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="611" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A611">
+        <v>3681</v>
+      </c>
+      <c r="B611">
+        <v>1</v>
+      </c>
+      <c r="C611">
+        <v>2</v>
+      </c>
+      <c r="D611">
+        <v>4</v>
+      </c>
+      <c r="E611">
+        <v>5</v>
+      </c>
+      <c r="F611">
+        <v>7</v>
+      </c>
+      <c r="G611">
+        <v>9</v>
+      </c>
+      <c r="H611">
+        <v>11</v>
+      </c>
+      <c r="I611">
+        <v>12</v>
+      </c>
+      <c r="J611">
+        <v>14</v>
+      </c>
+      <c r="K611">
+        <v>15</v>
+      </c>
+      <c r="L611">
+        <v>16</v>
+      </c>
+      <c r="M611">
+        <v>20</v>
+      </c>
+      <c r="N611">
+        <v>21</v>
+      </c>
+      <c r="O611">
+        <v>22</v>
+      </c>
+      <c r="P611">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="612" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A612">
+        <v>3682</v>
+      </c>
+      <c r="B612">
+        <v>1</v>
+      </c>
+      <c r="C612">
+        <v>2</v>
+      </c>
+      <c r="D612">
+        <v>4</v>
+      </c>
+      <c r="E612">
+        <v>5</v>
+      </c>
+      <c r="F612">
+        <v>7</v>
+      </c>
+      <c r="G612">
+        <v>9</v>
+      </c>
+      <c r="H612">
+        <v>10</v>
+      </c>
+      <c r="I612">
+        <v>11</v>
+      </c>
+      <c r="J612">
+        <v>12</v>
+      </c>
+      <c r="K612">
+        <v>13</v>
+      </c>
+      <c r="L612">
+        <v>17</v>
+      </c>
+      <c r="M612">
+        <v>18</v>
+      </c>
+      <c r="N612">
+        <v>21</v>
+      </c>
+      <c r="O612">
+        <v>22</v>
+      </c>
+      <c r="P612">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="613" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A613">
+        <v>3683</v>
+      </c>
+      <c r="B613">
+        <v>2</v>
+      </c>
+      <c r="C613">
+        <v>3</v>
+      </c>
+      <c r="D613">
+        <v>5</v>
+      </c>
+      <c r="E613">
+        <v>7</v>
+      </c>
+      <c r="F613">
+        <v>8</v>
+      </c>
+      <c r="G613">
+        <v>9</v>
+      </c>
+      <c r="H613">
+        <v>10</v>
+      </c>
+      <c r="I613">
+        <v>11</v>
+      </c>
+      <c r="J613">
+        <v>12</v>
+      </c>
+      <c r="K613">
+        <v>14</v>
+      </c>
+      <c r="L613">
+        <v>16</v>
+      </c>
+      <c r="M613">
+        <v>19</v>
+      </c>
+      <c r="N613">
+        <v>20</v>
+      </c>
+      <c r="O613">
+        <v>24</v>
+      </c>
+      <c r="P613">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="614" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A614">
+        <v>3684</v>
+      </c>
+      <c r="B614">
+        <v>1</v>
+      </c>
+      <c r="C614">
+        <v>3</v>
+      </c>
+      <c r="D614">
+        <v>5</v>
+      </c>
+      <c r="E614">
+        <v>6</v>
+      </c>
+      <c r="F614">
+        <v>9</v>
+      </c>
+      <c r="G614">
+        <v>10</v>
+      </c>
+      <c r="H614">
+        <v>11</v>
+      </c>
+      <c r="I614">
+        <v>12</v>
+      </c>
+      <c r="J614">
+        <v>13</v>
+      </c>
+      <c r="K614">
+        <v>17</v>
+      </c>
+      <c r="L614">
+        <v>18</v>
+      </c>
+      <c r="M614">
+        <v>19</v>
+      </c>
+      <c r="N614">
+        <v>20</v>
+      </c>
+      <c r="O614">
+        <v>21</v>
+      </c>
+      <c r="P614">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="615" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A615">
+        <v>3685</v>
+      </c>
+      <c r="B615">
+        <v>1</v>
+      </c>
+      <c r="C615">
+        <v>2</v>
+      </c>
+      <c r="D615">
+        <v>4</v>
+      </c>
+      <c r="E615">
+        <v>8</v>
+      </c>
+      <c r="F615">
+        <v>10</v>
+      </c>
+      <c r="G615">
+        <v>11</v>
+      </c>
+      <c r="H615">
+        <v>14</v>
+      </c>
+      <c r="I615">
+        <v>15</v>
+      </c>
+      <c r="J615">
+        <v>17</v>
+      </c>
+      <c r="K615">
+        <v>19</v>
+      </c>
+      <c r="L615">
+        <v>20</v>
+      </c>
+      <c r="M615">
+        <v>21</v>
+      </c>
+      <c r="N615">
+        <v>23</v>
+      </c>
+      <c r="O615">
+        <v>24</v>
+      </c>
+      <c r="P615">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="616" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A616">
+        <v>3686</v>
+      </c>
+      <c r="B616">
+        <v>1</v>
+      </c>
+      <c r="C616">
+        <v>2</v>
+      </c>
+      <c r="D616">
+        <v>4</v>
+      </c>
+      <c r="E616">
+        <v>5</v>
+      </c>
+      <c r="F616">
+        <v>6</v>
+      </c>
+      <c r="G616">
+        <v>8</v>
+      </c>
+      <c r="H616">
+        <v>9</v>
+      </c>
+      <c r="I616">
+        <v>10</v>
+      </c>
+      <c r="J616">
+        <v>13</v>
+      </c>
+      <c r="K616">
+        <v>15</v>
+      </c>
+      <c r="L616">
+        <v>18</v>
+      </c>
+      <c r="M616">
+        <v>19</v>
+      </c>
+      <c r="N616">
+        <v>23</v>
+      </c>
+      <c r="O616">
+        <v>24</v>
+      </c>
+      <c r="P616">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="617" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A617">
+        <v>3687</v>
+      </c>
+      <c r="B617">
+        <v>3</v>
+      </c>
+      <c r="C617">
+        <v>4</v>
+      </c>
+      <c r="D617">
+        <v>5</v>
+      </c>
+      <c r="E617">
+        <v>6</v>
+      </c>
+      <c r="F617">
+        <v>12</v>
+      </c>
+      <c r="G617">
+        <v>13</v>
+      </c>
+      <c r="H617">
+        <v>14</v>
+      </c>
+      <c r="I617">
+        <v>16</v>
+      </c>
+      <c r="J617">
+        <v>17</v>
+      </c>
+      <c r="K617">
+        <v>18</v>
+      </c>
+      <c r="L617">
+        <v>20</v>
+      </c>
+      <c r="M617">
+        <v>21</v>
+      </c>
+      <c r="N617">
+        <v>23</v>
+      </c>
+      <c r="O617">
+        <v>24</v>
+      </c>
+      <c r="P617">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="618" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A618">
+        <v>3688</v>
+      </c>
+      <c r="B618">
+        <v>1</v>
+      </c>
+      <c r="C618">
+        <v>2</v>
+      </c>
+      <c r="D618">
+        <v>3</v>
+      </c>
+      <c r="E618">
+        <v>4</v>
+      </c>
+      <c r="F618">
+        <v>5</v>
+      </c>
+      <c r="G618">
+        <v>6</v>
+      </c>
+      <c r="H618">
+        <v>7</v>
+      </c>
+      <c r="I618">
+        <v>11</v>
+      </c>
+      <c r="J618">
+        <v>12</v>
+      </c>
+      <c r="K618">
+        <v>16</v>
+      </c>
+      <c r="L618">
+        <v>17</v>
+      </c>
+      <c r="M618">
+        <v>19</v>
+      </c>
+      <c r="N618">
+        <v>21</v>
+      </c>
+      <c r="O618">
+        <v>24</v>
+      </c>
+      <c r="P618">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="619" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A619">
+        <v>3689</v>
+      </c>
+      <c r="B619">
+        <v>3</v>
+      </c>
+      <c r="C619">
+        <v>5</v>
+      </c>
+      <c r="D619">
+        <v>7</v>
+      </c>
+      <c r="E619">
+        <v>8</v>
+      </c>
+      <c r="F619">
+        <v>10</v>
+      </c>
+      <c r="G619">
+        <v>11</v>
+      </c>
+      <c r="H619">
+        <v>12</v>
+      </c>
+      <c r="I619">
+        <v>13</v>
+      </c>
+      <c r="J619">
+        <v>14</v>
+      </c>
+      <c r="K619">
+        <v>15</v>
+      </c>
+      <c r="L619">
+        <v>16</v>
+      </c>
+      <c r="M619">
+        <v>18</v>
+      </c>
+      <c r="N619">
+        <v>19</v>
+      </c>
+      <c r="O619">
+        <v>20</v>
+      </c>
+      <c r="P619">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="620" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A620">
+        <v>3690</v>
+      </c>
+      <c r="B620">
+        <v>2</v>
+      </c>
+      <c r="C620">
+        <v>5</v>
+      </c>
+      <c r="D620">
+        <v>6</v>
+      </c>
+      <c r="E620">
+        <v>7</v>
+      </c>
+      <c r="F620">
+        <v>8</v>
+      </c>
+      <c r="G620">
+        <v>9</v>
+      </c>
+      <c r="H620">
+        <v>12</v>
+      </c>
+      <c r="I620">
+        <v>15</v>
+      </c>
+      <c r="J620">
+        <v>18</v>
+      </c>
+      <c r="K620">
+        <v>19</v>
+      </c>
+      <c r="L620">
+        <v>20</v>
+      </c>
+      <c r="M620">
+        <v>21</v>
+      </c>
+      <c r="N620">
+        <v>22</v>
+      </c>
+      <c r="O620">
+        <v>24</v>
+      </c>
+      <c r="P620">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="621" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A621">
+        <v>3691</v>
+      </c>
+      <c r="B621">
+        <v>2</v>
+      </c>
+      <c r="C621">
+        <v>3</v>
+      </c>
+      <c r="D621">
+        <v>5</v>
+      </c>
+      <c r="E621">
+        <v>8</v>
+      </c>
+      <c r="F621">
+        <v>9</v>
+      </c>
+      <c r="G621">
+        <v>10</v>
+      </c>
+      <c r="H621">
+        <v>13</v>
+      </c>
+      <c r="I621">
+        <v>14</v>
+      </c>
+      <c r="J621">
+        <v>15</v>
+      </c>
+      <c r="K621">
+        <v>18</v>
+      </c>
+      <c r="L621">
+        <v>19</v>
+      </c>
+      <c r="M621">
+        <v>21</v>
+      </c>
+      <c r="N621">
+        <v>23</v>
+      </c>
+      <c r="O621">
+        <v>24</v>
+      </c>
+      <c r="P621">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="622" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A622">
+        <v>3692</v>
+      </c>
+      <c r="B622">
+        <v>2</v>
+      </c>
+      <c r="C622">
+        <v>3</v>
+      </c>
+      <c r="D622">
+        <v>5</v>
+      </c>
+      <c r="E622">
+        <v>6</v>
+      </c>
+      <c r="F622">
+        <v>7</v>
+      </c>
+      <c r="G622">
+        <v>9</v>
+      </c>
+      <c r="H622">
+        <v>10</v>
+      </c>
+      <c r="I622">
+        <v>13</v>
+      </c>
+      <c r="J622">
+        <v>14</v>
+      </c>
+      <c r="K622">
+        <v>15</v>
+      </c>
+      <c r="L622">
+        <v>19</v>
+      </c>
+      <c r="M622">
+        <v>20</v>
+      </c>
+      <c r="N622">
+        <v>23</v>
+      </c>
+      <c r="O622">
+        <v>24</v>
+      </c>
+      <c r="P622">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="623" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A623">
+        <v>3693</v>
+      </c>
+      <c r="B623">
+        <v>1</v>
+      </c>
+      <c r="C623">
+        <v>4</v>
+      </c>
+      <c r="D623">
+        <v>6</v>
+      </c>
+      <c r="E623">
+        <v>7</v>
+      </c>
+      <c r="F623">
+        <v>9</v>
+      </c>
+      <c r="G623">
+        <v>10</v>
+      </c>
+      <c r="H623">
+        <v>11</v>
+      </c>
+      <c r="I623">
+        <v>13</v>
+      </c>
+      <c r="J623">
+        <v>14</v>
+      </c>
+      <c r="K623">
+        <v>16</v>
+      </c>
+      <c r="L623">
+        <v>17</v>
+      </c>
+      <c r="M623">
+        <v>18</v>
+      </c>
+      <c r="N623">
+        <v>20</v>
+      </c>
+      <c r="O623">
+        <v>21</v>
+      </c>
+      <c r="P623">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="624" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A624">
+        <v>3694</v>
+      </c>
+      <c r="B624">
+        <v>2</v>
+      </c>
+      <c r="C624">
+        <v>4</v>
+      </c>
+      <c r="D624">
+        <v>5</v>
+      </c>
+      <c r="E624">
+        <v>7</v>
+      </c>
+      <c r="F624">
+        <v>8</v>
+      </c>
+      <c r="G624">
+        <v>9</v>
+      </c>
+      <c r="H624">
+        <v>13</v>
+      </c>
+      <c r="I624">
+        <v>14</v>
+      </c>
+      <c r="J624">
+        <v>17</v>
+      </c>
+      <c r="K624">
+        <v>18</v>
+      </c>
+      <c r="L624">
+        <v>19</v>
+      </c>
+      <c r="M624">
+        <v>20</v>
+      </c>
+      <c r="N624">
+        <v>22</v>
+      </c>
+      <c r="O624">
+        <v>23</v>
+      </c>
+      <c r="P624">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="625" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A625">
+        <v>3695</v>
+      </c>
+      <c r="B625">
+        <v>1</v>
+      </c>
+      <c r="C625">
+        <v>2</v>
+      </c>
+      <c r="D625">
+        <v>3</v>
+      </c>
+      <c r="E625">
+        <v>4</v>
+      </c>
+      <c r="F625">
+        <v>6</v>
+      </c>
+      <c r="G625">
+        <v>8</v>
+      </c>
+      <c r="H625">
+        <v>9</v>
+      </c>
+      <c r="I625">
+        <v>13</v>
+      </c>
+      <c r="J625">
+        <v>15</v>
+      </c>
+      <c r="K625">
+        <v>17</v>
+      </c>
+      <c r="L625">
+        <v>18</v>
+      </c>
+      <c r="M625">
+        <v>21</v>
+      </c>
+      <c r="N625">
+        <v>22</v>
+      </c>
+      <c r="O625">
+        <v>23</v>
+      </c>
+      <c r="P625">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="626" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A626">
+        <v>3696</v>
+      </c>
+      <c r="B626">
+        <v>2</v>
+      </c>
+      <c r="C626">
+        <v>3</v>
+      </c>
+      <c r="D626">
+        <v>5</v>
+      </c>
+      <c r="E626">
+        <v>6</v>
+      </c>
+      <c r="F626">
+        <v>7</v>
+      </c>
+      <c r="G626">
+        <v>9</v>
+      </c>
+      <c r="H626">
+        <v>11</v>
+      </c>
+      <c r="I626">
+        <v>13</v>
+      </c>
+      <c r="J626">
+        <v>15</v>
+      </c>
+      <c r="K626">
+        <v>16</v>
+      </c>
+      <c r="L626">
+        <v>17</v>
+      </c>
+      <c r="M626">
+        <v>19</v>
+      </c>
+      <c r="N626">
+        <v>21</v>
+      </c>
+      <c r="O626">
+        <v>23</v>
+      </c>
+      <c r="P626">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="627" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A627">
+        <v>3697</v>
+      </c>
+      <c r="B627">
+        <v>1</v>
+      </c>
+      <c r="C627">
+        <v>5</v>
+      </c>
+      <c r="D627">
+        <v>6</v>
+      </c>
+      <c r="E627">
+        <v>7</v>
+      </c>
+      <c r="F627">
+        <v>9</v>
+      </c>
+      <c r="G627">
+        <v>10</v>
+      </c>
+      <c r="H627">
+        <v>13</v>
+      </c>
+      <c r="I627">
+        <v>15</v>
+      </c>
+      <c r="J627">
+        <v>17</v>
+      </c>
+      <c r="K627">
+        <v>18</v>
+      </c>
+      <c r="L627">
+        <v>19</v>
+      </c>
+      <c r="M627">
+        <v>20</v>
+      </c>
+      <c r="N627">
+        <v>21</v>
+      </c>
+      <c r="O627">
+        <v>24</v>
+      </c>
+      <c r="P627">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="628" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A628">
+        <v>3698</v>
+      </c>
+      <c r="B628">
+        <v>1</v>
+      </c>
+      <c r="C628">
+        <v>3</v>
+      </c>
+      <c r="D628">
+        <v>5</v>
+      </c>
+      <c r="E628">
+        <v>6</v>
+      </c>
+      <c r="F628">
+        <v>7</v>
+      </c>
+      <c r="G628">
+        <v>8</v>
+      </c>
+      <c r="H628">
+        <v>9</v>
+      </c>
+      <c r="I628">
+        <v>10</v>
+      </c>
+      <c r="J628">
+        <v>12</v>
+      </c>
+      <c r="K628">
+        <v>13</v>
+      </c>
+      <c r="L628">
+        <v>16</v>
+      </c>
+      <c r="M628">
+        <v>18</v>
+      </c>
+      <c r="N628">
+        <v>20</v>
+      </c>
+      <c r="O628">
+        <v>21</v>
+      </c>
+      <c r="P628">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="629" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A629">
+        <v>3699</v>
+      </c>
+      <c r="B629">
+        <v>1</v>
+      </c>
+      <c r="C629">
+        <v>2</v>
+      </c>
+      <c r="D629">
+        <v>3</v>
+      </c>
+      <c r="E629">
+        <v>5</v>
+      </c>
+      <c r="F629">
+        <v>6</v>
+      </c>
+      <c r="G629">
+        <v>8</v>
+      </c>
+      <c r="H629">
+        <v>9</v>
+      </c>
+      <c r="I629">
+        <v>11</v>
+      </c>
+      <c r="J629">
+        <v>14</v>
+      </c>
+      <c r="K629">
+        <v>18</v>
+      </c>
+      <c r="L629">
+        <v>20</v>
+      </c>
+      <c r="M629">
+        <v>21</v>
+      </c>
+      <c r="N629">
+        <v>22</v>
+      </c>
+      <c r="O629">
+        <v>24</v>
+      </c>
+      <c r="P629">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="630" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A630">
+        <v>3700</v>
+      </c>
+      <c r="B630">
+        <v>1</v>
+      </c>
+      <c r="C630">
+        <v>3</v>
+      </c>
+      <c r="D630">
+        <v>7</v>
+      </c>
+      <c r="E630">
+        <v>8</v>
+      </c>
+      <c r="F630">
+        <v>9</v>
+      </c>
+      <c r="G630">
+        <v>10</v>
+      </c>
+      <c r="H630">
+        <v>12</v>
+      </c>
+      <c r="I630">
+        <v>13</v>
+      </c>
+      <c r="J630">
+        <v>14</v>
+      </c>
+      <c r="K630">
+        <v>17</v>
+      </c>
+      <c r="L630">
+        <v>18</v>
+      </c>
+      <c r="M630">
+        <v>19</v>
+      </c>
+      <c r="N630">
+        <v>20</v>
+      </c>
+      <c r="O630">
+        <v>23</v>
+      </c>
+      <c r="P630">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="631" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A631">
+        <v>3701</v>
+      </c>
+      <c r="B631">
+        <v>1</v>
+      </c>
+      <c r="C631">
+        <v>2</v>
+      </c>
+      <c r="D631">
+        <v>4</v>
+      </c>
+      <c r="E631">
+        <v>7</v>
+      </c>
+      <c r="F631">
+        <v>8</v>
+      </c>
+      <c r="G631">
+        <v>9</v>
+      </c>
+      <c r="H631">
+        <v>10</v>
+      </c>
+      <c r="I631">
+        <v>12</v>
+      </c>
+      <c r="J631">
+        <v>13</v>
+      </c>
+      <c r="K631">
+        <v>14</v>
+      </c>
+      <c r="L631">
+        <v>17</v>
+      </c>
+      <c r="M631">
+        <v>22</v>
+      </c>
+      <c r="N631">
+        <v>23</v>
+      </c>
+      <c r="O631">
+        <v>24</v>
+      </c>
+      <c r="P631">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="632" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A632">
+        <v>3702</v>
+      </c>
+      <c r="B632">
+        <v>2</v>
+      </c>
+      <c r="C632">
+        <v>3</v>
+      </c>
+      <c r="D632">
+        <v>5</v>
+      </c>
+      <c r="E632">
+        <v>9</v>
+      </c>
+      <c r="F632">
+        <v>13</v>
+      </c>
+      <c r="G632">
+        <v>14</v>
+      </c>
+      <c r="H632">
+        <v>15</v>
+      </c>
+      <c r="I632">
+        <v>16</v>
+      </c>
+      <c r="J632">
+        <v>17</v>
+      </c>
+      <c r="K632">
+        <v>18</v>
+      </c>
+      <c r="L632">
+        <v>20</v>
+      </c>
+      <c r="M632">
+        <v>21</v>
+      </c>
+      <c r="N632">
+        <v>22</v>
+      </c>
+      <c r="O632">
+        <v>23</v>
+      </c>
+      <c r="P632">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="633" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A633">
+        <v>3703</v>
+      </c>
+      <c r="B633">
+        <v>1</v>
+      </c>
+      <c r="C633">
+        <v>3</v>
+      </c>
+      <c r="D633">
+        <v>5</v>
+      </c>
+      <c r="E633">
+        <v>7</v>
+      </c>
+      <c r="F633">
+        <v>8</v>
+      </c>
+      <c r="G633">
+        <v>9</v>
+      </c>
+      <c r="H633">
+        <v>10</v>
+      </c>
+      <c r="I633">
+        <v>14</v>
+      </c>
+      <c r="J633">
+        <v>15</v>
+      </c>
+      <c r="K633">
+        <v>17</v>
+      </c>
+      <c r="L633">
+        <v>21</v>
+      </c>
+      <c r="M633">
+        <v>22</v>
+      </c>
+      <c r="N633">
+        <v>23</v>
+      </c>
+      <c r="O633">
+        <v>24</v>
+      </c>
+      <c r="P633">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="634" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A634">
+        <v>3704</v>
+      </c>
+      <c r="B634">
+        <v>1</v>
+      </c>
+      <c r="C634">
+        <v>3</v>
+      </c>
+      <c r="D634">
+        <v>4</v>
+      </c>
+      <c r="E634">
+        <v>9</v>
+      </c>
+      <c r="F634">
+        <v>10</v>
+      </c>
+      <c r="G634">
+        <v>11</v>
+      </c>
+      <c r="H634">
+        <v>12</v>
+      </c>
+      <c r="I634">
+        <v>13</v>
+      </c>
+      <c r="J634">
+        <v>14</v>
+      </c>
+      <c r="K634">
+        <v>15</v>
+      </c>
+      <c r="L634">
+        <v>19</v>
+      </c>
+      <c r="M634">
+        <v>20</v>
+      </c>
+      <c r="N634">
+        <v>22</v>
+      </c>
+      <c r="O634">
+        <v>23</v>
+      </c>
+      <c r="P634">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="635" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A635">
+        <v>3705</v>
+      </c>
+      <c r="B635">
+        <v>1</v>
+      </c>
+      <c r="C635">
+        <v>3</v>
+      </c>
+      <c r="D635">
+        <v>4</v>
+      </c>
+      <c r="E635">
+        <v>6</v>
+      </c>
+      <c r="F635">
+        <v>8</v>
+      </c>
+      <c r="G635">
+        <v>10</v>
+      </c>
+      <c r="H635">
+        <v>14</v>
+      </c>
+      <c r="I635">
+        <v>15</v>
+      </c>
+      <c r="J635">
+        <v>16</v>
+      </c>
+      <c r="K635">
+        <v>18</v>
+      </c>
+      <c r="L635">
+        <v>20</v>
+      </c>
+      <c r="M635">
+        <v>21</v>
+      </c>
+      <c r="N635">
+        <v>22</v>
+      </c>
+      <c r="O635">
+        <v>24</v>
+      </c>
+      <c r="P635">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="636" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A636">
+        <v>3706</v>
+      </c>
+      <c r="B636">
+        <v>1</v>
+      </c>
+      <c r="C636">
+        <v>4</v>
+      </c>
+      <c r="D636">
+        <v>6</v>
+      </c>
+      <c r="E636">
+        <v>8</v>
+      </c>
+      <c r="F636">
+        <v>9</v>
+      </c>
+      <c r="G636">
+        <v>10</v>
+      </c>
+      <c r="H636">
+        <v>12</v>
+      </c>
+      <c r="I636">
+        <v>14</v>
+      </c>
+      <c r="J636">
+        <v>15</v>
+      </c>
+      <c r="K636">
+        <v>16</v>
+      </c>
+      <c r="L636">
+        <v>18</v>
+      </c>
+      <c r="M636">
+        <v>21</v>
+      </c>
+      <c r="N636">
+        <v>22</v>
+      </c>
+      <c r="O636">
+        <v>24</v>
+      </c>
+      <c r="P636">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="637" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A637">
+        <v>3707</v>
+      </c>
+      <c r="B637">
+        <v>1</v>
+      </c>
+      <c r="C637">
+        <v>2</v>
+      </c>
+      <c r="D637">
+        <v>3</v>
+      </c>
+      <c r="E637">
+        <v>7</v>
+      </c>
+      <c r="F637">
+        <v>8</v>
+      </c>
+      <c r="G637">
+        <v>9</v>
+      </c>
+      <c r="H637">
+        <v>10</v>
+      </c>
+      <c r="I637">
+        <v>13</v>
+      </c>
+      <c r="J637">
+        <v>14</v>
+      </c>
+      <c r="K637">
+        <v>18</v>
+      </c>
+      <c r="L637">
+        <v>20</v>
+      </c>
+      <c r="M637">
+        <v>21</v>
+      </c>
+      <c r="N637">
+        <v>22</v>
+      </c>
+      <c r="O637">
+        <v>23</v>
+      </c>
+      <c r="P637">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="638" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A638">
+        <v>3708</v>
+      </c>
+      <c r="B638">
+        <v>1</v>
+      </c>
+      <c r="C638">
+        <v>2</v>
+      </c>
+      <c r="D638">
+        <v>4</v>
+      </c>
+      <c r="E638">
+        <v>5</v>
+      </c>
+      <c r="F638">
+        <v>6</v>
+      </c>
+      <c r="G638">
+        <v>8</v>
+      </c>
+      <c r="H638">
+        <v>9</v>
+      </c>
+      <c r="I638">
+        <v>12</v>
+      </c>
+      <c r="J638">
+        <v>16</v>
+      </c>
+      <c r="K638">
+        <v>17</v>
+      </c>
+      <c r="L638">
+        <v>18</v>
+      </c>
+      <c r="M638">
+        <v>19</v>
+      </c>
+      <c r="N638">
+        <v>21</v>
+      </c>
+      <c r="O638">
+        <v>23</v>
+      </c>
+      <c r="P638">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="639" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A639">
+        <v>3709</v>
+      </c>
+      <c r="B639">
+        <v>1</v>
+      </c>
+      <c r="C639">
+        <v>4</v>
+      </c>
+      <c r="D639">
+        <v>6</v>
+      </c>
+      <c r="E639">
+        <v>7</v>
+      </c>
+      <c r="F639">
+        <v>9</v>
+      </c>
+      <c r="G639">
+        <v>10</v>
+      </c>
+      <c r="H639">
+        <v>11</v>
+      </c>
+      <c r="I639">
+        <v>14</v>
+      </c>
+      <c r="J639">
+        <v>15</v>
+      </c>
+      <c r="K639">
+        <v>18</v>
+      </c>
+      <c r="L639">
+        <v>19</v>
+      </c>
+      <c r="M639">
+        <v>20</v>
+      </c>
+      <c r="N639">
+        <v>23</v>
+      </c>
+      <c r="O639">
+        <v>24</v>
+      </c>
+      <c r="P639">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="640" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A640">
+        <v>3710</v>
+      </c>
+      <c r="B640">
+        <v>1</v>
+      </c>
+      <c r="C640">
+        <v>2</v>
+      </c>
+      <c r="D640">
+        <v>3</v>
+      </c>
+      <c r="E640">
+        <v>4</v>
+      </c>
+      <c r="F640">
+        <v>5</v>
+      </c>
+      <c r="G640">
+        <v>6</v>
+      </c>
+      <c r="H640">
+        <v>9</v>
+      </c>
+      <c r="I640">
+        <v>12</v>
+      </c>
+      <c r="J640">
+        <v>13</v>
+      </c>
+      <c r="K640">
+        <v>14</v>
+      </c>
+      <c r="L640">
+        <v>15</v>
+      </c>
+      <c r="M640">
+        <v>16</v>
+      </c>
+      <c r="N640">
+        <v>17</v>
+      </c>
+      <c r="O640">
+        <v>18</v>
+      </c>
+      <c r="P640">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="641" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A641">
+        <v>3711</v>
+      </c>
+      <c r="B641">
+        <v>1</v>
+      </c>
+      <c r="C641">
+        <v>5</v>
+      </c>
+      <c r="D641">
+        <v>6</v>
+      </c>
+      <c r="E641">
+        <v>8</v>
+      </c>
+      <c r="F641">
+        <v>9</v>
+      </c>
+      <c r="G641">
+        <v>10</v>
+      </c>
+      <c r="H641">
+        <v>12</v>
+      </c>
+      <c r="I641">
+        <v>13</v>
+      </c>
+      <c r="J641">
+        <v>15</v>
+      </c>
+      <c r="K641">
+        <v>16</v>
+      </c>
+      <c r="L641">
+        <v>17</v>
+      </c>
+      <c r="M641">
+        <v>20</v>
+      </c>
+      <c r="N641">
+        <v>22</v>
+      </c>
+      <c r="O641">
+        <v>24</v>
+      </c>
+      <c r="P641">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="642" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A642">
+        <v>3712</v>
+      </c>
+      <c r="B642">
+        <v>1</v>
+      </c>
+      <c r="C642">
+        <v>3</v>
+      </c>
+      <c r="D642">
+        <v>4</v>
+      </c>
+      <c r="E642">
+        <v>6</v>
+      </c>
+      <c r="F642">
+        <v>13</v>
+      </c>
+      <c r="G642">
+        <v>14</v>
+      </c>
+      <c r="H642">
+        <v>15</v>
+      </c>
+      <c r="I642">
+        <v>16</v>
+      </c>
+      <c r="J642">
+        <v>18</v>
+      </c>
+      <c r="K642">
+        <v>19</v>
+      </c>
+      <c r="L642">
+        <v>20</v>
+      </c>
+      <c r="M642">
+        <v>21</v>
+      </c>
+      <c r="N642">
+        <v>22</v>
+      </c>
+      <c r="O642">
+        <v>23</v>
+      </c>
+      <c r="P642">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="643" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A643">
+        <v>3713</v>
+      </c>
+      <c r="B643">
+        <v>2</v>
+      </c>
+      <c r="C643">
+        <v>4</v>
+      </c>
+      <c r="D643">
+        <v>5</v>
+      </c>
+      <c r="E643">
+        <v>6</v>
+      </c>
+      <c r="F643">
+        <v>7</v>
+      </c>
+      <c r="G643">
+        <v>8</v>
+      </c>
+      <c r="H643">
+        <v>9</v>
+      </c>
+      <c r="I643">
+        <v>11</v>
+      </c>
+      <c r="J643">
+        <v>12</v>
+      </c>
+      <c r="K643">
+        <v>13</v>
+      </c>
+      <c r="L643">
+        <v>14</v>
+      </c>
+      <c r="M643">
+        <v>15</v>
+      </c>
+      <c r="N643">
+        <v>19</v>
+      </c>
+      <c r="O643">
+        <v>20</v>
+      </c>
+      <c r="P643">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="644" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A644">
+        <v>3714</v>
+      </c>
+      <c r="B644">
+        <v>3</v>
+      </c>
+      <c r="C644">
+        <v>4</v>
+      </c>
+      <c r="D644">
+        <v>5</v>
+      </c>
+      <c r="E644">
+        <v>6</v>
+      </c>
+      <c r="F644">
+        <v>9</v>
+      </c>
+      <c r="G644">
+        <v>10</v>
+      </c>
+      <c r="H644">
+        <v>11</v>
+      </c>
+      <c r="I644">
+        <v>12</v>
+      </c>
+      <c r="J644">
+        <v>13</v>
+      </c>
+      <c r="K644">
+        <v>14</v>
+      </c>
+      <c r="L644">
+        <v>15</v>
+      </c>
+      <c r="M644">
+        <v>16</v>
+      </c>
+      <c r="N644">
+        <v>18</v>
+      </c>
+      <c r="O644">
+        <v>19</v>
+      </c>
+      <c r="P644">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="645" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A645">
+        <v>3715</v>
+      </c>
+      <c r="B645">
+        <v>3</v>
+      </c>
+      <c r="C645">
+        <v>5</v>
+      </c>
+      <c r="D645">
+        <v>6</v>
+      </c>
+      <c r="E645">
+        <v>9</v>
+      </c>
+      <c r="F645">
+        <v>11</v>
+      </c>
+      <c r="G645">
+        <v>12</v>
+      </c>
+      <c r="H645">
+        <v>14</v>
+      </c>
+      <c r="I645">
+        <v>16</v>
+      </c>
+      <c r="J645">
+        <v>18</v>
+      </c>
+      <c r="K645">
+        <v>20</v>
+      </c>
+      <c r="L645">
+        <v>21</v>
+      </c>
+      <c r="M645">
+        <v>22</v>
+      </c>
+      <c r="N645">
+        <v>23</v>
+      </c>
+      <c r="O645">
+        <v>24</v>
+      </c>
+      <c r="P645">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="646" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A646">
+        <v>3716</v>
+      </c>
+      <c r="B646">
+        <v>1</v>
+      </c>
+      <c r="C646">
+        <v>2</v>
+      </c>
+      <c r="D646">
+        <v>4</v>
+      </c>
+      <c r="E646">
+        <v>5</v>
+      </c>
+      <c r="F646">
+        <v>7</v>
+      </c>
+      <c r="G646">
+        <v>11</v>
+      </c>
+      <c r="H646">
+        <v>12</v>
+      </c>
+      <c r="I646">
+        <v>15</v>
+      </c>
+      <c r="J646">
+        <v>17</v>
+      </c>
+      <c r="K646">
+        <v>18</v>
+      </c>
+      <c r="L646">
+        <v>21</v>
+      </c>
+      <c r="M646">
+        <v>22</v>
+      </c>
+      <c r="N646">
+        <v>23</v>
+      </c>
+      <c r="O646">
+        <v>24</v>
+      </c>
+      <c r="P646">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C92CDE8829F3C7438DCCB0991C30EAAE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36cf41eecaf38ba1d849a0c8dd067090">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="3e38fcf2-aa96-4a2c-865b-c3abba01ba51" xmlns:ns3="4455b8ba-124f-46d5-aaaa-9813efd83d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="023f68b2d27389a617bf935a3f0e17ad" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -31108,15 +32967,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -31128,6 +32978,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B637BD-743B-452C-A85E-33AF8B93F052}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C5B8C5-4575-4105-836C-9C4A6674A14B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -31147,14 +33005,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B637BD-743B-452C-A85E-33AF8B93F052}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0328C38C-FE97-4791-8469-4B5D9CCC5D08}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
atualizando excel loterias e carrossel
</commit_message>
<xml_diff>
--- a/LoteriasExcel/Lotofacil_edt2.xlsx
+++ b/LoteriasExcel/Lotofacil_edt2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Dropbox\! 000 ByPass\Pessoal\99_Loterias\0 - Loterias-Inteligentes\LoteriasExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8DFD9C6-FA04-4BD7-9470-029CF90C30EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771FF0FE-D1B5-41AD-A143-175009050442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57540" yWindow="120" windowWidth="19515" windowHeight="14565" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
+    <workbookView xWindow="67755" yWindow="1935" windowWidth="19770" windowHeight="11130" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
   </bookViews>
   <sheets>
     <sheet name="LOTOFÁCIL" sheetId="3" r:id="rId1"/>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69BEFC42-DD13-4DE0-B2AD-D0F44AF8189C}">
-  <dimension ref="A1:P652"/>
+  <dimension ref="A1:P659"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="17" max="17" width="11.6640625" customWidth="1"/>
@@ -32988,103 +32988,453 @@
       </c>
     </row>
     <row r="651" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A651" s="5">
+      <c r="A651">
         <v>3721</v>
       </c>
-      <c r="B651" s="6">
-        <v>1</v>
-      </c>
-      <c r="C651" s="6">
-        <v>3</v>
-      </c>
-      <c r="D651" s="6">
-        <v>4</v>
-      </c>
-      <c r="E651" s="6">
-        <v>5</v>
-      </c>
-      <c r="F651" s="6">
-        <v>7</v>
-      </c>
-      <c r="G651" s="6">
-        <v>8</v>
-      </c>
-      <c r="H651" s="6">
-        <v>10</v>
-      </c>
-      <c r="I651" s="6">
-        <v>11</v>
-      </c>
-      <c r="J651" s="6">
-        <v>12</v>
-      </c>
-      <c r="K651" s="6">
-        <v>14</v>
-      </c>
-      <c r="L651" s="6">
-        <v>15</v>
-      </c>
-      <c r="M651" s="6">
-        <v>20</v>
-      </c>
-      <c r="N651" s="6">
-        <v>21</v>
-      </c>
-      <c r="O651" s="6">
-        <v>23</v>
-      </c>
-      <c r="P651" s="6">
+      <c r="B651">
+        <v>1</v>
+      </c>
+      <c r="C651">
+        <v>3</v>
+      </c>
+      <c r="D651">
+        <v>4</v>
+      </c>
+      <c r="E651">
+        <v>5</v>
+      </c>
+      <c r="F651">
+        <v>7</v>
+      </c>
+      <c r="G651">
+        <v>8</v>
+      </c>
+      <c r="H651">
+        <v>10</v>
+      </c>
+      <c r="I651">
+        <v>11</v>
+      </c>
+      <c r="J651">
+        <v>12</v>
+      </c>
+      <c r="K651">
+        <v>14</v>
+      </c>
+      <c r="L651">
+        <v>15</v>
+      </c>
+      <c r="M651">
+        <v>20</v>
+      </c>
+      <c r="N651">
+        <v>21</v>
+      </c>
+      <c r="O651">
+        <v>23</v>
+      </c>
+      <c r="P651">
         <v>24</v>
       </c>
     </row>
     <row r="652" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A652" s="5">
+      <c r="A652">
         <v>3722</v>
       </c>
-      <c r="B652" s="6">
-        <v>2</v>
-      </c>
-      <c r="C652" s="6">
-        <v>3</v>
-      </c>
-      <c r="D652" s="6">
-        <v>5</v>
-      </c>
-      <c r="E652" s="6">
-        <v>6</v>
-      </c>
-      <c r="F652" s="6">
-        <v>9</v>
-      </c>
-      <c r="G652" s="6">
-        <v>10</v>
-      </c>
-      <c r="H652" s="6">
-        <v>11</v>
-      </c>
-      <c r="I652" s="6">
-        <v>12</v>
-      </c>
-      <c r="J652" s="6">
-        <v>13</v>
-      </c>
-      <c r="K652" s="6">
-        <v>14</v>
-      </c>
-      <c r="L652" s="6">
-        <v>15</v>
-      </c>
-      <c r="M652" s="6">
-        <v>17</v>
-      </c>
-      <c r="N652" s="6">
-        <v>19</v>
-      </c>
-      <c r="O652" s="6">
-        <v>20</v>
-      </c>
-      <c r="P652" s="6">
-        <v>23</v>
+      <c r="B652">
+        <v>2</v>
+      </c>
+      <c r="C652">
+        <v>3</v>
+      </c>
+      <c r="D652">
+        <v>5</v>
+      </c>
+      <c r="E652">
+        <v>6</v>
+      </c>
+      <c r="F652">
+        <v>9</v>
+      </c>
+      <c r="G652">
+        <v>10</v>
+      </c>
+      <c r="H652">
+        <v>11</v>
+      </c>
+      <c r="I652">
+        <v>12</v>
+      </c>
+      <c r="J652">
+        <v>13</v>
+      </c>
+      <c r="K652">
+        <v>14</v>
+      </c>
+      <c r="L652">
+        <v>15</v>
+      </c>
+      <c r="M652">
+        <v>17</v>
+      </c>
+      <c r="N652">
+        <v>19</v>
+      </c>
+      <c r="O652">
+        <v>20</v>
+      </c>
+      <c r="P652">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="653" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A653" s="5">
+        <v>3723</v>
+      </c>
+      <c r="B653" s="6">
+        <v>2</v>
+      </c>
+      <c r="C653" s="6">
+        <v>4</v>
+      </c>
+      <c r="D653" s="6">
+        <v>5</v>
+      </c>
+      <c r="E653" s="6">
+        <v>6</v>
+      </c>
+      <c r="F653" s="6">
+        <v>7</v>
+      </c>
+      <c r="G653" s="6">
+        <v>10</v>
+      </c>
+      <c r="H653" s="6">
+        <v>12</v>
+      </c>
+      <c r="I653" s="6">
+        <v>15</v>
+      </c>
+      <c r="J653" s="6">
+        <v>17</v>
+      </c>
+      <c r="K653" s="6">
+        <v>18</v>
+      </c>
+      <c r="L653" s="6">
+        <v>19</v>
+      </c>
+      <c r="M653" s="6">
+        <v>20</v>
+      </c>
+      <c r="N653" s="6">
+        <v>22</v>
+      </c>
+      <c r="O653" s="6">
+        <v>23</v>
+      </c>
+      <c r="P653" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="654" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A654" s="5">
+        <v>3724</v>
+      </c>
+      <c r="B654" s="6">
+        <v>1</v>
+      </c>
+      <c r="C654" s="6">
+        <v>2</v>
+      </c>
+      <c r="D654" s="6">
+        <v>3</v>
+      </c>
+      <c r="E654" s="6">
+        <v>5</v>
+      </c>
+      <c r="F654" s="6">
+        <v>6</v>
+      </c>
+      <c r="G654" s="6">
+        <v>7</v>
+      </c>
+      <c r="H654" s="6">
+        <v>12</v>
+      </c>
+      <c r="I654" s="6">
+        <v>15</v>
+      </c>
+      <c r="J654" s="6">
+        <v>16</v>
+      </c>
+      <c r="K654" s="6">
+        <v>17</v>
+      </c>
+      <c r="L654" s="6">
+        <v>19</v>
+      </c>
+      <c r="M654" s="6">
+        <v>21</v>
+      </c>
+      <c r="N654" s="6">
+        <v>22</v>
+      </c>
+      <c r="O654" s="6">
+        <v>24</v>
+      </c>
+      <c r="P654" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="655" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A655" s="5">
+        <v>3725</v>
+      </c>
+      <c r="B655" s="6">
+        <v>1</v>
+      </c>
+      <c r="C655" s="6">
+        <v>2</v>
+      </c>
+      <c r="D655" s="6">
+        <v>4</v>
+      </c>
+      <c r="E655" s="6">
+        <v>5</v>
+      </c>
+      <c r="F655" s="6">
+        <v>6</v>
+      </c>
+      <c r="G655" s="6">
+        <v>8</v>
+      </c>
+      <c r="H655" s="6">
+        <v>11</v>
+      </c>
+      <c r="I655" s="6">
+        <v>13</v>
+      </c>
+      <c r="J655" s="6">
+        <v>14</v>
+      </c>
+      <c r="K655" s="6">
+        <v>16</v>
+      </c>
+      <c r="L655" s="6">
+        <v>17</v>
+      </c>
+      <c r="M655" s="6">
+        <v>19</v>
+      </c>
+      <c r="N655" s="6">
+        <v>21</v>
+      </c>
+      <c r="O655" s="6">
+        <v>24</v>
+      </c>
+      <c r="P655" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="656" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A656" s="5">
+        <v>3726</v>
+      </c>
+      <c r="B656" s="6">
+        <v>2</v>
+      </c>
+      <c r="C656" s="6">
+        <v>5</v>
+      </c>
+      <c r="D656" s="6">
+        <v>6</v>
+      </c>
+      <c r="E656" s="6">
+        <v>7</v>
+      </c>
+      <c r="F656" s="6">
+        <v>10</v>
+      </c>
+      <c r="G656" s="6">
+        <v>13</v>
+      </c>
+      <c r="H656" s="6">
+        <v>14</v>
+      </c>
+      <c r="I656" s="6">
+        <v>17</v>
+      </c>
+      <c r="J656" s="6">
+        <v>18</v>
+      </c>
+      <c r="K656" s="6">
+        <v>19</v>
+      </c>
+      <c r="L656" s="6">
+        <v>20</v>
+      </c>
+      <c r="M656" s="6">
+        <v>21</v>
+      </c>
+      <c r="N656" s="6">
+        <v>22</v>
+      </c>
+      <c r="O656" s="6">
+        <v>24</v>
+      </c>
+      <c r="P656" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="657" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A657" s="5">
+        <v>3727</v>
+      </c>
+      <c r="B657" s="6">
+        <v>1</v>
+      </c>
+      <c r="C657" s="6">
+        <v>2</v>
+      </c>
+      <c r="D657" s="6">
+        <v>3</v>
+      </c>
+      <c r="E657" s="6">
+        <v>4</v>
+      </c>
+      <c r="F657" s="6">
+        <v>5</v>
+      </c>
+      <c r="G657" s="6">
+        <v>9</v>
+      </c>
+      <c r="H657" s="6">
+        <v>10</v>
+      </c>
+      <c r="I657" s="6">
+        <v>11</v>
+      </c>
+      <c r="J657" s="6">
+        <v>13</v>
+      </c>
+      <c r="K657" s="6">
+        <v>14</v>
+      </c>
+      <c r="L657" s="6">
+        <v>16</v>
+      </c>
+      <c r="M657" s="6">
+        <v>18</v>
+      </c>
+      <c r="N657" s="6">
+        <v>19</v>
+      </c>
+      <c r="O657" s="6">
+        <v>22</v>
+      </c>
+      <c r="P657" s="6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="658" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A658" s="5">
+        <v>3728</v>
+      </c>
+      <c r="B658" s="6">
+        <v>1</v>
+      </c>
+      <c r="C658" s="6">
+        <v>2</v>
+      </c>
+      <c r="D658" s="6">
+        <v>3</v>
+      </c>
+      <c r="E658" s="6">
+        <v>6</v>
+      </c>
+      <c r="F658" s="6">
+        <v>7</v>
+      </c>
+      <c r="G658" s="6">
+        <v>8</v>
+      </c>
+      <c r="H658" s="6">
+        <v>10</v>
+      </c>
+      <c r="I658" s="6">
+        <v>11</v>
+      </c>
+      <c r="J658" s="6">
+        <v>16</v>
+      </c>
+      <c r="K658" s="6">
+        <v>17</v>
+      </c>
+      <c r="L658" s="6">
+        <v>19</v>
+      </c>
+      <c r="M658" s="6">
+        <v>21</v>
+      </c>
+      <c r="N658" s="6">
+        <v>22</v>
+      </c>
+      <c r="O658" s="6">
+        <v>23</v>
+      </c>
+      <c r="P658" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="659" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A659" s="5">
+        <v>3729</v>
+      </c>
+      <c r="B659" s="6">
+        <v>1</v>
+      </c>
+      <c r="C659" s="6">
+        <v>2</v>
+      </c>
+      <c r="D659" s="6">
+        <v>3</v>
+      </c>
+      <c r="E659" s="6">
+        <v>5</v>
+      </c>
+      <c r="F659" s="6">
+        <v>6</v>
+      </c>
+      <c r="G659" s="6">
+        <v>11</v>
+      </c>
+      <c r="H659" s="6">
+        <v>12</v>
+      </c>
+      <c r="I659" s="6">
+        <v>13</v>
+      </c>
+      <c r="J659" s="6">
+        <v>14</v>
+      </c>
+      <c r="K659" s="6">
+        <v>15</v>
+      </c>
+      <c r="L659" s="6">
+        <v>16</v>
+      </c>
+      <c r="M659" s="6">
+        <v>18</v>
+      </c>
+      <c r="N659" s="6">
+        <v>20</v>
+      </c>
+      <c r="O659" s="6">
+        <v>21</v>
+      </c>
+      <c r="P659" s="6">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -33093,6 +33443,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2025-08-17T04:03:58+00:00</AtualizadoPeloTimerJobEm>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C92CDE8829F3C7438DCCB0991C30EAAE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36cf41eecaf38ba1d849a0c8dd067090">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="3e38fcf2-aa96-4a2c-865b-c3abba01ba51" xmlns:ns3="4455b8ba-124f-46d5-aaaa-9813efd83d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="023f68b2d27389a617bf935a3f0e17ad" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -33260,16 +33620,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2025-08-17T04:03:58+00:00</AtualizadoPeloTimerJobEm>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -33280,6 +33630,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0328C38C-FE97-4791-8469-4B5D9CCC5D08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4455b8ba-124f-46d5-aaaa-9813efd83d1e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C5B8C5-4575-4105-836C-9C4A6674A14B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -33299,17 +33660,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0328C38C-FE97-4791-8469-4B5D9CCC5D08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4455b8ba-124f-46d5-aaaa-9813efd83d1e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B637BD-743B-452C-A85E-33AF8B93F052}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
atualizando arquivos excel loterias
</commit_message>
<xml_diff>
--- a/LoteriasExcel/Lotofacil_edt2.xlsx
+++ b/LoteriasExcel/Lotofacil_edt2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Dropbox\! 000 ByPass\Pessoal\99_Loterias\0 - Loterias-Inteligentes\LoteriasExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C2741F-47FF-45D5-BD74-02B30854E050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{871C2593-12F7-4AEC-A723-7D7C9243430C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58335" yWindow="735" windowWidth="26985" windowHeight="7695" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
+    <workbookView xWindow="2940" yWindow="2940" windowWidth="22395" windowHeight="10358" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
   </bookViews>
   <sheets>
     <sheet name="LOTOFÁCIL" sheetId="3" r:id="rId1"/>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69BEFC42-DD13-4DE0-B2AD-D0F44AF8189C}">
-  <dimension ref="A1:P666"/>
+  <dimension ref="A1:P677"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="17" max="17" width="11.6640625" customWidth="1"/>
@@ -33588,203 +33588,753 @@
       </c>
     </row>
     <row r="663" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A663" s="5">
+      <c r="A663">
         <v>3733</v>
       </c>
-      <c r="B663" s="6">
-        <v>1</v>
-      </c>
-      <c r="C663" s="6">
-        <v>2</v>
-      </c>
-      <c r="D663" s="6">
-        <v>3</v>
-      </c>
-      <c r="E663" s="6">
-        <v>5</v>
-      </c>
-      <c r="F663" s="6">
-        <v>7</v>
-      </c>
-      <c r="G663" s="6">
-        <v>10</v>
-      </c>
-      <c r="H663" s="6">
-        <v>11</v>
-      </c>
-      <c r="I663" s="6">
-        <v>12</v>
-      </c>
-      <c r="J663" s="6">
-        <v>13</v>
-      </c>
-      <c r="K663" s="6">
-        <v>14</v>
-      </c>
-      <c r="L663" s="6">
-        <v>16</v>
-      </c>
-      <c r="M663" s="6">
-        <v>17</v>
-      </c>
-      <c r="N663" s="6">
-        <v>19</v>
-      </c>
-      <c r="O663" s="6">
-        <v>22</v>
-      </c>
-      <c r="P663" s="6">
+      <c r="B663">
+        <v>1</v>
+      </c>
+      <c r="C663">
+        <v>2</v>
+      </c>
+      <c r="D663">
+        <v>3</v>
+      </c>
+      <c r="E663">
+        <v>5</v>
+      </c>
+      <c r="F663">
+        <v>7</v>
+      </c>
+      <c r="G663">
+        <v>10</v>
+      </c>
+      <c r="H663">
+        <v>11</v>
+      </c>
+      <c r="I663">
+        <v>12</v>
+      </c>
+      <c r="J663">
+        <v>13</v>
+      </c>
+      <c r="K663">
+        <v>14</v>
+      </c>
+      <c r="L663">
+        <v>16</v>
+      </c>
+      <c r="M663">
+        <v>17</v>
+      </c>
+      <c r="N663">
+        <v>19</v>
+      </c>
+      <c r="O663">
+        <v>22</v>
+      </c>
+      <c r="P663">
         <v>25</v>
       </c>
     </row>
     <row r="664" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A664" s="5">
+      <c r="A664">
         <v>3734</v>
       </c>
-      <c r="B664" s="6">
-        <v>2</v>
-      </c>
-      <c r="C664" s="6">
-        <v>3</v>
-      </c>
-      <c r="D664" s="6">
-        <v>5</v>
-      </c>
-      <c r="E664" s="6">
-        <v>8</v>
-      </c>
-      <c r="F664" s="6">
-        <v>10</v>
-      </c>
-      <c r="G664" s="6">
-        <v>12</v>
-      </c>
-      <c r="H664" s="6">
-        <v>13</v>
-      </c>
-      <c r="I664" s="6">
-        <v>14</v>
-      </c>
-      <c r="J664" s="6">
-        <v>15</v>
-      </c>
-      <c r="K664" s="6">
-        <v>16</v>
-      </c>
-      <c r="L664" s="6">
-        <v>17</v>
-      </c>
-      <c r="M664" s="6">
-        <v>19</v>
-      </c>
-      <c r="N664" s="6">
-        <v>22</v>
-      </c>
-      <c r="O664" s="6">
-        <v>23</v>
-      </c>
-      <c r="P664" s="6">
+      <c r="B664">
+        <v>2</v>
+      </c>
+      <c r="C664">
+        <v>3</v>
+      </c>
+      <c r="D664">
+        <v>5</v>
+      </c>
+      <c r="E664">
+        <v>8</v>
+      </c>
+      <c r="F664">
+        <v>10</v>
+      </c>
+      <c r="G664">
+        <v>12</v>
+      </c>
+      <c r="H664">
+        <v>13</v>
+      </c>
+      <c r="I664">
+        <v>14</v>
+      </c>
+      <c r="J664">
+        <v>15</v>
+      </c>
+      <c r="K664">
+        <v>16</v>
+      </c>
+      <c r="L664">
+        <v>17</v>
+      </c>
+      <c r="M664">
+        <v>19</v>
+      </c>
+      <c r="N664">
+        <v>22</v>
+      </c>
+      <c r="O664">
+        <v>23</v>
+      </c>
+      <c r="P664">
         <v>25</v>
       </c>
     </row>
     <row r="665" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A665" s="5">
+      <c r="A665">
         <v>3735</v>
       </c>
-      <c r="B665" s="6">
-        <v>3</v>
-      </c>
-      <c r="C665" s="6">
-        <v>5</v>
-      </c>
-      <c r="D665" s="6">
-        <v>7</v>
-      </c>
-      <c r="E665" s="6">
-        <v>12</v>
-      </c>
-      <c r="F665" s="6">
-        <v>14</v>
-      </c>
-      <c r="G665" s="6">
-        <v>15</v>
-      </c>
-      <c r="H665" s="6">
-        <v>16</v>
-      </c>
-      <c r="I665" s="6">
-        <v>17</v>
-      </c>
-      <c r="J665" s="6">
-        <v>18</v>
-      </c>
-      <c r="K665" s="6">
-        <v>20</v>
-      </c>
-      <c r="L665" s="6">
-        <v>21</v>
-      </c>
-      <c r="M665" s="6">
-        <v>22</v>
-      </c>
-      <c r="N665" s="6">
-        <v>23</v>
-      </c>
-      <c r="O665" s="6">
-        <v>24</v>
-      </c>
-      <c r="P665" s="6">
+      <c r="B665">
+        <v>3</v>
+      </c>
+      <c r="C665">
+        <v>5</v>
+      </c>
+      <c r="D665">
+        <v>7</v>
+      </c>
+      <c r="E665">
+        <v>12</v>
+      </c>
+      <c r="F665">
+        <v>14</v>
+      </c>
+      <c r="G665">
+        <v>15</v>
+      </c>
+      <c r="H665">
+        <v>16</v>
+      </c>
+      <c r="I665">
+        <v>17</v>
+      </c>
+      <c r="J665">
+        <v>18</v>
+      </c>
+      <c r="K665">
+        <v>20</v>
+      </c>
+      <c r="L665">
+        <v>21</v>
+      </c>
+      <c r="M665">
+        <v>22</v>
+      </c>
+      <c r="N665">
+        <v>23</v>
+      </c>
+      <c r="O665">
+        <v>24</v>
+      </c>
+      <c r="P665">
         <v>25</v>
       </c>
     </row>
     <row r="666" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A666" s="5">
+      <c r="A666">
         <v>3736</v>
       </c>
-      <c r="B666" s="6">
-        <v>3</v>
-      </c>
-      <c r="C666" s="6">
-        <v>4</v>
-      </c>
-      <c r="D666" s="6">
-        <v>6</v>
-      </c>
-      <c r="E666" s="6">
-        <v>7</v>
-      </c>
-      <c r="F666" s="6">
-        <v>8</v>
-      </c>
-      <c r="G666" s="6">
-        <v>9</v>
-      </c>
-      <c r="H666" s="6">
-        <v>11</v>
-      </c>
-      <c r="I666" s="6">
-        <v>12</v>
-      </c>
-      <c r="J666" s="6">
-        <v>14</v>
-      </c>
-      <c r="K666" s="6">
-        <v>17</v>
-      </c>
-      <c r="L666" s="6">
-        <v>18</v>
-      </c>
-      <c r="M666" s="6">
-        <v>19</v>
-      </c>
-      <c r="N666" s="6">
-        <v>21</v>
-      </c>
-      <c r="O666" s="6">
-        <v>22</v>
-      </c>
-      <c r="P666" s="6">
-        <v>23</v>
+      <c r="B666">
+        <v>3</v>
+      </c>
+      <c r="C666">
+        <v>4</v>
+      </c>
+      <c r="D666">
+        <v>6</v>
+      </c>
+      <c r="E666">
+        <v>7</v>
+      </c>
+      <c r="F666">
+        <v>8</v>
+      </c>
+      <c r="G666">
+        <v>9</v>
+      </c>
+      <c r="H666">
+        <v>11</v>
+      </c>
+      <c r="I666">
+        <v>12</v>
+      </c>
+      <c r="J666">
+        <v>14</v>
+      </c>
+      <c r="K666">
+        <v>17</v>
+      </c>
+      <c r="L666">
+        <v>18</v>
+      </c>
+      <c r="M666">
+        <v>19</v>
+      </c>
+      <c r="N666">
+        <v>21</v>
+      </c>
+      <c r="O666">
+        <v>22</v>
+      </c>
+      <c r="P666">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="667" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A667" s="5">
+        <v>3737</v>
+      </c>
+      <c r="B667" s="6">
+        <v>2</v>
+      </c>
+      <c r="C667" s="6">
+        <v>3</v>
+      </c>
+      <c r="D667" s="6">
+        <v>5</v>
+      </c>
+      <c r="E667" s="6">
+        <v>6</v>
+      </c>
+      <c r="F667" s="6">
+        <v>8</v>
+      </c>
+      <c r="G667" s="6">
+        <v>9</v>
+      </c>
+      <c r="H667" s="6">
+        <v>11</v>
+      </c>
+      <c r="I667" s="6">
+        <v>12</v>
+      </c>
+      <c r="J667" s="6">
+        <v>13</v>
+      </c>
+      <c r="K667" s="6">
+        <v>14</v>
+      </c>
+      <c r="L667" s="6">
+        <v>15</v>
+      </c>
+      <c r="M667" s="6">
+        <v>17</v>
+      </c>
+      <c r="N667" s="6">
+        <v>22</v>
+      </c>
+      <c r="O667" s="6">
+        <v>23</v>
+      </c>
+      <c r="P667" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="668" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A668" s="5">
+        <v>3738</v>
+      </c>
+      <c r="B668" s="6">
+        <v>2</v>
+      </c>
+      <c r="C668" s="6">
+        <v>3</v>
+      </c>
+      <c r="D668" s="6">
+        <v>4</v>
+      </c>
+      <c r="E668" s="6">
+        <v>5</v>
+      </c>
+      <c r="F668" s="6">
+        <v>7</v>
+      </c>
+      <c r="G668" s="6">
+        <v>8</v>
+      </c>
+      <c r="H668" s="6">
+        <v>10</v>
+      </c>
+      <c r="I668" s="6">
+        <v>11</v>
+      </c>
+      <c r="J668" s="6">
+        <v>13</v>
+      </c>
+      <c r="K668" s="6">
+        <v>14</v>
+      </c>
+      <c r="L668" s="6">
+        <v>17</v>
+      </c>
+      <c r="M668" s="6">
+        <v>18</v>
+      </c>
+      <c r="N668" s="6">
+        <v>20</v>
+      </c>
+      <c r="O668" s="6">
+        <v>23</v>
+      </c>
+      <c r="P668" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="669" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A669" s="5">
+        <v>3739</v>
+      </c>
+      <c r="B669" s="6">
+        <v>1</v>
+      </c>
+      <c r="C669" s="6">
+        <v>4</v>
+      </c>
+      <c r="D669" s="6">
+        <v>5</v>
+      </c>
+      <c r="E669" s="6">
+        <v>6</v>
+      </c>
+      <c r="F669" s="6">
+        <v>9</v>
+      </c>
+      <c r="G669" s="6">
+        <v>11</v>
+      </c>
+      <c r="H669" s="6">
+        <v>13</v>
+      </c>
+      <c r="I669" s="6">
+        <v>15</v>
+      </c>
+      <c r="J669" s="6">
+        <v>16</v>
+      </c>
+      <c r="K669" s="6">
+        <v>18</v>
+      </c>
+      <c r="L669" s="6">
+        <v>19</v>
+      </c>
+      <c r="M669" s="6">
+        <v>20</v>
+      </c>
+      <c r="N669" s="6">
+        <v>23</v>
+      </c>
+      <c r="O669" s="6">
+        <v>24</v>
+      </c>
+      <c r="P669" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="670" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A670" s="5">
+        <v>3740</v>
+      </c>
+      <c r="B670" s="6">
+        <v>1</v>
+      </c>
+      <c r="C670" s="6">
+        <v>2</v>
+      </c>
+      <c r="D670" s="6">
+        <v>5</v>
+      </c>
+      <c r="E670" s="6">
+        <v>6</v>
+      </c>
+      <c r="F670" s="6">
+        <v>8</v>
+      </c>
+      <c r="G670" s="6">
+        <v>9</v>
+      </c>
+      <c r="H670" s="6">
+        <v>11</v>
+      </c>
+      <c r="I670" s="6">
+        <v>12</v>
+      </c>
+      <c r="J670" s="6">
+        <v>13</v>
+      </c>
+      <c r="K670" s="6">
+        <v>15</v>
+      </c>
+      <c r="L670" s="6">
+        <v>16</v>
+      </c>
+      <c r="M670" s="6">
+        <v>17</v>
+      </c>
+      <c r="N670" s="6">
+        <v>20</v>
+      </c>
+      <c r="O670" s="6">
+        <v>21</v>
+      </c>
+      <c r="P670" s="6">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="671" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A671" s="5">
+        <v>3741</v>
+      </c>
+      <c r="B671" s="6">
+        <v>2</v>
+      </c>
+      <c r="C671" s="6">
+        <v>3</v>
+      </c>
+      <c r="D671" s="6">
+        <v>4</v>
+      </c>
+      <c r="E671" s="6">
+        <v>5</v>
+      </c>
+      <c r="F671" s="6">
+        <v>9</v>
+      </c>
+      <c r="G671" s="6">
+        <v>11</v>
+      </c>
+      <c r="H671" s="6">
+        <v>12</v>
+      </c>
+      <c r="I671" s="6">
+        <v>14</v>
+      </c>
+      <c r="J671" s="6">
+        <v>15</v>
+      </c>
+      <c r="K671" s="6">
+        <v>16</v>
+      </c>
+      <c r="L671" s="6">
+        <v>18</v>
+      </c>
+      <c r="M671" s="6">
+        <v>20</v>
+      </c>
+      <c r="N671" s="6">
+        <v>21</v>
+      </c>
+      <c r="O671" s="6">
+        <v>22</v>
+      </c>
+      <c r="P671" s="6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="672" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A672" s="5">
+        <v>3742</v>
+      </c>
+      <c r="B672" s="6">
+        <v>1</v>
+      </c>
+      <c r="C672" s="6">
+        <v>4</v>
+      </c>
+      <c r="D672" s="6">
+        <v>5</v>
+      </c>
+      <c r="E672" s="6">
+        <v>6</v>
+      </c>
+      <c r="F672" s="6">
+        <v>9</v>
+      </c>
+      <c r="G672" s="6">
+        <v>10</v>
+      </c>
+      <c r="H672" s="6">
+        <v>12</v>
+      </c>
+      <c r="I672" s="6">
+        <v>13</v>
+      </c>
+      <c r="J672" s="6">
+        <v>14</v>
+      </c>
+      <c r="K672" s="6">
+        <v>15</v>
+      </c>
+      <c r="L672" s="6">
+        <v>16</v>
+      </c>
+      <c r="M672" s="6">
+        <v>19</v>
+      </c>
+      <c r="N672" s="6">
+        <v>20</v>
+      </c>
+      <c r="O672" s="6">
+        <v>21</v>
+      </c>
+      <c r="P672" s="6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="673" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A673" s="5">
+        <v>3743</v>
+      </c>
+      <c r="B673" s="6">
+        <v>2</v>
+      </c>
+      <c r="C673" s="6">
+        <v>3</v>
+      </c>
+      <c r="D673" s="6">
+        <v>4</v>
+      </c>
+      <c r="E673" s="6">
+        <v>5</v>
+      </c>
+      <c r="F673" s="6">
+        <v>9</v>
+      </c>
+      <c r="G673" s="6">
+        <v>10</v>
+      </c>
+      <c r="H673" s="6">
+        <v>11</v>
+      </c>
+      <c r="I673" s="6">
+        <v>13</v>
+      </c>
+      <c r="J673" s="6">
+        <v>15</v>
+      </c>
+      <c r="K673" s="6">
+        <v>18</v>
+      </c>
+      <c r="L673" s="6">
+        <v>19</v>
+      </c>
+      <c r="M673" s="6">
+        <v>20</v>
+      </c>
+      <c r="N673" s="6">
+        <v>21</v>
+      </c>
+      <c r="O673" s="6">
+        <v>23</v>
+      </c>
+      <c r="P673" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="674" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A674" s="5">
+        <v>3744</v>
+      </c>
+      <c r="B674" s="6">
+        <v>1</v>
+      </c>
+      <c r="C674" s="6">
+        <v>2</v>
+      </c>
+      <c r="D674" s="6">
+        <v>3</v>
+      </c>
+      <c r="E674" s="6">
+        <v>5</v>
+      </c>
+      <c r="F674" s="6">
+        <v>7</v>
+      </c>
+      <c r="G674" s="6">
+        <v>10</v>
+      </c>
+      <c r="H674" s="6">
+        <v>14</v>
+      </c>
+      <c r="I674" s="6">
+        <v>16</v>
+      </c>
+      <c r="J674" s="6">
+        <v>17</v>
+      </c>
+      <c r="K674" s="6">
+        <v>18</v>
+      </c>
+      <c r="L674" s="6">
+        <v>20</v>
+      </c>
+      <c r="M674" s="6">
+        <v>21</v>
+      </c>
+      <c r="N674" s="6">
+        <v>22</v>
+      </c>
+      <c r="O674" s="6">
+        <v>23</v>
+      </c>
+      <c r="P674" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="675" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A675" s="5">
+        <v>3745</v>
+      </c>
+      <c r="B675" s="6">
+        <v>1</v>
+      </c>
+      <c r="C675" s="6">
+        <v>2</v>
+      </c>
+      <c r="D675" s="6">
+        <v>4</v>
+      </c>
+      <c r="E675" s="6">
+        <v>5</v>
+      </c>
+      <c r="F675" s="6">
+        <v>6</v>
+      </c>
+      <c r="G675" s="6">
+        <v>7</v>
+      </c>
+      <c r="H675" s="6">
+        <v>8</v>
+      </c>
+      <c r="I675" s="6">
+        <v>9</v>
+      </c>
+      <c r="J675" s="6">
+        <v>10</v>
+      </c>
+      <c r="K675" s="6">
+        <v>12</v>
+      </c>
+      <c r="L675" s="6">
+        <v>13</v>
+      </c>
+      <c r="M675" s="6">
+        <v>19</v>
+      </c>
+      <c r="N675" s="6">
+        <v>21</v>
+      </c>
+      <c r="O675" s="6">
+        <v>22</v>
+      </c>
+      <c r="P675" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="676" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A676" s="5">
+        <v>3746</v>
+      </c>
+      <c r="B676" s="6">
+        <v>1</v>
+      </c>
+      <c r="C676" s="6">
+        <v>3</v>
+      </c>
+      <c r="D676" s="6">
+        <v>4</v>
+      </c>
+      <c r="E676" s="6">
+        <v>6</v>
+      </c>
+      <c r="F676" s="6">
+        <v>7</v>
+      </c>
+      <c r="G676" s="6">
+        <v>8</v>
+      </c>
+      <c r="H676" s="6">
+        <v>9</v>
+      </c>
+      <c r="I676" s="6">
+        <v>10</v>
+      </c>
+      <c r="J676" s="6">
+        <v>14</v>
+      </c>
+      <c r="K676" s="6">
+        <v>15</v>
+      </c>
+      <c r="L676" s="6">
+        <v>17</v>
+      </c>
+      <c r="M676" s="6">
+        <v>18</v>
+      </c>
+      <c r="N676" s="6">
+        <v>21</v>
+      </c>
+      <c r="O676" s="6">
+        <v>22</v>
+      </c>
+      <c r="P676" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="677" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A677" s="5">
+        <v>3747</v>
+      </c>
+      <c r="B677" s="6">
+        <v>1</v>
+      </c>
+      <c r="C677" s="6">
+        <v>2</v>
+      </c>
+      <c r="D677" s="6">
+        <v>4</v>
+      </c>
+      <c r="E677" s="6">
+        <v>5</v>
+      </c>
+      <c r="F677" s="6">
+        <v>6</v>
+      </c>
+      <c r="G677" s="6">
+        <v>8</v>
+      </c>
+      <c r="H677" s="6">
+        <v>9</v>
+      </c>
+      <c r="I677" s="6">
+        <v>11</v>
+      </c>
+      <c r="J677" s="6">
+        <v>12</v>
+      </c>
+      <c r="K677" s="6">
+        <v>13</v>
+      </c>
+      <c r="L677" s="6">
+        <v>18</v>
+      </c>
+      <c r="M677" s="6">
+        <v>19</v>
+      </c>
+      <c r="N677" s="6">
+        <v>21</v>
+      </c>
+      <c r="O677" s="6">
+        <v>24</v>
+      </c>
+      <c r="P677" s="6">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -33793,16 +34343,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2025-08-17T04:03:58+00:00</AtualizadoPeloTimerJobEm>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C92CDE8829F3C7438DCCB0991C30EAAE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36cf41eecaf38ba1d849a0c8dd067090">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="3e38fcf2-aa96-4a2c-865b-c3abba01ba51" xmlns:ns3="4455b8ba-124f-46d5-aaaa-9813efd83d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="023f68b2d27389a617bf935a3f0e17ad" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -33970,6 +34510,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2025-08-17T04:03:58+00:00</AtualizadoPeloTimerJobEm>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -33980,17 +34530,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0328C38C-FE97-4791-8469-4B5D9CCC5D08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4455b8ba-124f-46d5-aaaa-9813efd83d1e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C5B8C5-4575-4105-836C-9C4A6674A14B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34010,6 +34549,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0328C38C-FE97-4791-8469-4B5D9CCC5D08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4455b8ba-124f-46d5-aaaa-9813efd83d1e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B637BD-743B-452C-A85E-33AF8B93F052}">
   <ds:schemaRefs>

</xml_diff>